<commit_message>
feat: add new LEDs to handleliste
</commit_message>
<xml_diff>
--- a/Handleliste-hardware.xlsx
+++ b/Handleliste-hardware.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="53">
   <si>
     <t xml:space="preserve">Komponent</t>
   </si>
@@ -157,22 +157,28 @@
     <t xml:space="preserve">https://www.digikey.no/no/products/detail/on-shore-technology-inc/USB-A1HSW6/2677750</t>
   </si>
   <si>
-    <t xml:space="preserve">LED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cree LED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JK3030AWT-P-B65EA0000-N0000001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.no/no/products/detail/cree-led/JK3030AWT-P-B65EA0000-N0000001/8020361</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uvisst</t>
-  </si>
-  <si>
     <t xml:space="preserve">Motstand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED (Grønn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lite-On Inc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LTST-C193KGKT-5A </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/no/products/detail/liteon/LTST-C193KGKT-5A/2356242</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED (Rød)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LTST-C193KRKT-5A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/no/products/detail/liteon/LTST-C193KRKT-5A/2356244</t>
   </si>
 </sst>
 </file>
@@ -550,7 +556,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:G14"/>
+  <dimension ref="A2:G1048576"/>
   <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="74.57"/>
@@ -794,28 +800,54 @@
       <c r="B13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="G13" s="1" t="e">
+      <c r="G13" s="1" t="n">
         <f aca="false">F13*3</f>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F14" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="1" t="n">
+        <f aca="false">F14*3</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
+      <c r="C15" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" s="1" t="n">
+        <f aca="false">F15*3</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E3" r:id="rId1" display="https://www.digikey.no/no/products/detail/stmicroelectronics/STM32U5G7VJT6Q/21700656"/>

</xml_diff>

<commit_message>
docs: add FPGA, VGA-port and SRAM to shopping list
Oscillator got updated, the initial entry was wrong.
</commit_message>
<xml_diff>
--- a/Handleliste-hardware.xlsx
+++ b/Handleliste-hardware.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="86">
   <si>
     <t xml:space="preserve">Komponent</t>
   </si>
@@ -193,58 +193,91 @@
     <t xml:space="preserve">Oscillator (100MHz, FPGA)</t>
   </si>
   <si>
+    <t xml:space="preserve">Connor Winfield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CWX813-100.0M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/no/products/detail/connor-winfield/CWX813-100-0M/695541</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flash (FPGA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GigaDevice Semiconductor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GD25F128FS2GR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/no/products/detail/gigadevice-semiconductor-hk-limited/GD25F128FS2GR/20531633</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nedtransformator (Power Supply)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texas Instruments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPS54294PWP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/no/products/detail/texas-instruments/TPS54294PWP/2812688</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRAM (FPGA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integrated Silicon Solution Inc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IS66WVH16M8DBLL-100B1LI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/no/products/detail/issi-integrated-silicon-solution-inc/IS66WVH16M8DBLL-100B1LI/6202025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FPGA DEBUG Header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FPGA pin header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCU Debug Header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCU pin header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FPGA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XC7A100T-2FTG256I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/no/products/detail/amd/XC7A100T-2FTG256I/3925791?s=N4IgTCBcDaIBoGEDsBBAjABgwFQLRgDFsBxMAVgDYBJEAXQF8g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VGA-port</t>
+  </si>
+  <si>
     <t xml:space="preserve">Amphenol ICC</t>
   </si>
   <si>
     <t xml:space="preserve">L77HDE15SD1CH4RHNVGA</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.digikey.no/no/products/detail/amphenol-cs-commercial-products/L77HDE15SD1CH4RHNVGA/25816614</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flash (FPGA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GigaDevice Semiconductor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GD25F128FS2GR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.no/no/products/detail/gigadevice-semiconductor-hk-limited/GD25F128FS2GR/20531633</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nedtransformator (Power Supply)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Texas Instruments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TPS54294PWP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.no/no/products/detail/texas-instruments/TPS54294PWP/2812688</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRAM (FPGA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FPGA DEBUG Header</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FPGA pin header</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCU Debug Header</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCU pin header</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FPGA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">VGA-port</t>
+    <t xml:space="preserve">https://www.digikey.no/en/products/detail/amphenol-cs-commercial-products/L77HDE15SD1CH4RHNVGA/25816614</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jumper 2x1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jumper cap</t>
   </si>
 </sst>
 </file>
@@ -348,7 +381,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -374,6 +407,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -637,7 +674,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="28.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="32.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="151"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.86"/>
@@ -1011,16 +1048,25 @@
         <v>68</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>39</v>
+        <v>69</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F20" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G20" s="1" t="n">
         <f aca="false">F20*3</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G21" s="1" t="n">
         <f aca="false">F21*3</f>
@@ -1029,7 +1075,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G22" s="1" t="n">
         <f aca="false">F22*3</f>
@@ -1038,7 +1084,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G23" s="1" t="n">
         <f aca="false">F23*3</f>
@@ -1047,7 +1093,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G24" s="1" t="n">
         <f aca="false">F24*3</f>
@@ -1056,20 +1102,65 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F25" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G25" s="1" t="n">
         <f aca="false">F25*3</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>83</v>
       </c>
       <c r="G26" s="1" t="n">
         <f aca="false">F26*3</f>
         <v>0</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F27" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="G27" s="1" t="n">
+        <f aca="false">F27*3</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F28" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" s="1" t="n">
+        <f aca="false">F28*3</f>
+        <v>12</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1083,6 +1174,8 @@
     <hyperlink ref="E8" r:id="rId6" display="https://no.mouser.com/ProductDetail/Displaytech/DT043CTFT-IPS-PTS?qs=sGAEpiMZZMt7dcPGmvnkBgpwamjCGwcHY0DbS%252B%2F%2FaodWnRIGq7eMYg%3D%3D"/>
     <hyperlink ref="E10" r:id="rId7" display="https://www.digikey.no/no/products/detail/phihong-usa/PSA15R-150P6-R/5247157"/>
     <hyperlink ref="E11" r:id="rId8" display="https://www.digikey.no/no/products/detail/stmicroelectronics/STLINK-V3MINIE/16284301"/>
+    <hyperlink ref="E17" r:id="rId9" display="https://www.digikey.no/no/products/detail/connor-winfield/CWX813-100-0M/695541"/>
+    <hyperlink ref="E20" r:id="rId10" display="https://www.digikey.no/no/products/detail/issi-integrated-silicon-solution-inc/IS66WVH16M8DBLL-100B1LI/6202025"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
feat: add remaining components and prices to Handleliste
We've now got all (probably) hardware stuff in the shopping list.
The total price lies at 9909 NOK.

Should probably check that we've actually included all components, but
there's a good chance we actually do have them all.
</commit_message>
<xml_diff>
--- a/Handleliste-hardware.xlsx
+++ b/Handleliste-hardware.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="161">
   <si>
     <t xml:space="preserve">Komponent</t>
   </si>
@@ -247,16 +247,40 @@
     <t xml:space="preserve">https://www.digikey.no/no/products/detail/issi-integrated-silicon-solution-inc/IS66WVH16M8DBLL-100B1LI/6202025 </t>
   </si>
   <si>
-    <t xml:space="preserve">FPGA DEBUG Header</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FPGA pin header</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCU Debug Header</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCU pin header</t>
+    <t xml:space="preserve">FPGA Debug Header (2x7, 2.54mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sullins Connector Solutions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SBH11-PBPC-D07-ST-BK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/en/products/detail/sullins-connector-solutions/SBH11-PBPC-D07-ST-BK/1990063</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FPGA pin header (2x7, 2.54mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCU Debug Header (2x7, 1.27mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CNC Tech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1175-1630-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/en/products/detail/cnc-tech/3220-14-0100-00/3883664</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCU pin header (1x8, 2.54mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Würth Elektronik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/en/products/detail/w%C3%BCrth-elektronik/61300811121/4846839</t>
   </si>
   <si>
     <t xml:space="preserve">FPGA </t>
@@ -283,12 +307,21 @@
     <t xml:space="preserve">https://www.digikey.no/en/products/detail/amphenol-cs-commercial-products/L77HDE15SD1CH4RHNVGA/25816614 </t>
   </si>
   <si>
-    <t xml:space="preserve">Jumper 2x1</t>
+    <t xml:space="preserve">PWR Header Pin (2x1, 2.54mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/no/products/detail/w%C3%BCrth-elektronik/61300211121/4846823</t>
   </si>
   <si>
     <t xml:space="preserve">Jumper cap</t>
   </si>
   <si>
+    <t xml:space="preserve">S9337-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/en/products/detail/sullins-connector-solutions/QPC02SXGN-RC/2618262</t>
+  </si>
+  <si>
     <t xml:space="preserve">Motstander</t>
   </si>
   <si>
@@ -448,10 +481,19 @@
     <t xml:space="preserve">Spoler</t>
   </si>
   <si>
+    <t xml:space="preserve">1,5u</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.digikey.no/no/products/detail/murata-electronics/LQM21PN1R5MC0D/1788280</t>
   </si>
   <si>
+    <t xml:space="preserve">2,2u</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.digikey.no/no/products/detail/murata-electronics/DFE201210U-2R2M-P2/7595453 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,3u</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.digikey.no/no/products/detail/murata-electronics/LQM21PN3R3MGRD/4359175 </t>
@@ -566,11 +608,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -578,15 +620,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -594,7 +636,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -853,230 +895,230 @@
   <dimension ref="A2:K1048576"/>
   <sheetFormatPr defaultColWidth="8.55859375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="32.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="33.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="5.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="9.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="6.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="28.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="32.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="33.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="5.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="6.67"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="0" t="s">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="0" t="s">
+      <c r="E2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="H2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="J2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="K2" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" s="0" t="n">
+      <c r="F3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="1" t="n">
         <f aca="false">F3*3</f>
         <v>3</v>
       </c>
-      <c r="H3" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="I3" s="0" t="n">
+      <c r="H3" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I3" s="1" t="n">
         <v>173.7</v>
       </c>
-      <c r="J3" s="0" t="n">
+      <c r="J3" s="1" t="n">
         <f aca="false">H3*I3</f>
         <v>521.1</v>
       </c>
-      <c r="K3" s="2" t="b">
+      <c r="K3" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="0" t="n">
+      <c r="F4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="1" t="n">
         <f aca="false">F4*3</f>
         <v>3</v>
       </c>
-      <c r="H4" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="I4" s="0" t="n">
+      <c r="H4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I4" s="1" t="n">
         <v>29.03</v>
       </c>
-      <c r="J4" s="0" t="n">
+      <c r="J4" s="1" t="n">
         <f aca="false">H4*I4</f>
         <v>87.09</v>
       </c>
-      <c r="K4" s="2" t="b">
+      <c r="K4" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="0" t="n">
+      <c r="F5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="1" t="n">
         <f aca="false">F5*3</f>
         <v>3</v>
       </c>
-      <c r="H5" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="I5" s="0" t="n">
+      <c r="H5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" s="1" t="n">
         <v>10.09</v>
       </c>
-      <c r="J5" s="0" t="n">
+      <c r="J5" s="1" t="n">
         <f aca="false">H5*I5</f>
         <v>30.27</v>
       </c>
-      <c r="K5" s="2" t="b">
+      <c r="K5" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>1492</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" s="0" t="n">
+      <c r="F6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="1" t="n">
         <f aca="false">F6*3</f>
         <v>3</v>
       </c>
-      <c r="H6" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="I6" s="0" t="n">
+      <c r="H6" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I6" s="1" t="n">
         <v>30.05</v>
       </c>
-      <c r="J6" s="0" t="n">
+      <c r="J6" s="1" t="n">
         <f aca="false">H6*I6</f>
         <v>90.15</v>
       </c>
-      <c r="K6" s="2" t="b">
+      <c r="K6" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>26</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="0" t="n">
+      <c r="F7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="1" t="n">
         <f aca="false">F7*3</f>
         <v>3</v>
       </c>
-      <c r="H7" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="I7" s="0" t="n">
+      <c r="H7" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="1" t="n">
         <v>37.59</v>
       </c>
-      <c r="J7" s="0" t="n">
+      <c r="J7" s="1" t="n">
         <f aca="false">H7*I7</f>
         <v>112.77</v>
       </c>
-      <c r="K7" s="2" t="b">
+      <c r="K7" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D8" s="4" t="s">
@@ -1085,1513 +1127,1615 @@
       <c r="E8" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F8" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="0" t="n">
+      <c r="F8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="1" t="n">
         <f aca="false">F8*3</f>
         <v>3</v>
       </c>
-      <c r="H8" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="I8" s="0" t="n">
+      <c r="H8" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" s="1" t="n">
         <v>542.36</v>
       </c>
-      <c r="J8" s="0" t="n">
+      <c r="J8" s="1" t="n">
         <f aca="false">H8*I8</f>
         <v>1627.08</v>
       </c>
-      <c r="K8" s="2" t="b">
+      <c r="K8" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>34</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F9" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="0" t="n">
+      <c r="F9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="1" t="n">
         <f aca="false">F9*3</f>
         <v>3</v>
       </c>
-      <c r="H9" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="I9" s="0" t="n">
+      <c r="H9" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I9" s="1" t="n">
         <v>5.3</v>
       </c>
-      <c r="J9" s="0" t="n">
+      <c r="J9" s="1" t="n">
         <f aca="false">H9*I9</f>
         <v>15.9</v>
       </c>
-      <c r="K9" s="2" t="b">
+      <c r="K9" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>38</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="F10" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="0" t="n">
+      <c r="F10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="1" t="n">
         <f aca="false">F10*3</f>
         <v>3</v>
       </c>
-      <c r="H10" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="I10" s="0" t="n">
+      <c r="H10" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="1" t="n">
         <v>93.52</v>
       </c>
-      <c r="J10" s="0" t="n">
+      <c r="J10" s="1" t="n">
         <f aca="false">H10*I10</f>
         <v>280.56</v>
       </c>
-      <c r="K10" s="2" t="b">
+      <c r="K10" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="1" t="s">
         <v>41</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="F11" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J11" s="0" t="n">
+      <c r="J11" s="1" t="n">
         <f aca="false">H11*I11</f>
         <v>0</v>
       </c>
-      <c r="K11" s="2" t="b">
+      <c r="K11" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>46</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="0" t="n">
+      <c r="F12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="1" t="n">
         <f aca="false">F12*3</f>
         <v>3</v>
       </c>
-      <c r="H12" s="0" t="n">
+      <c r="H12" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I12" s="0" t="n">
+      <c r="I12" s="1" t="n">
         <v>5.09</v>
       </c>
-      <c r="J12" s="0" t="n">
+      <c r="J12" s="1" t="n">
         <f aca="false">H12*I12</f>
         <v>20.36</v>
       </c>
-      <c r="K12" s="2" t="b">
+      <c r="K12" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="G13" s="0" t="n">
+      <c r="G13" s="1" t="n">
         <f aca="false">F13*3</f>
         <v>0</v>
       </c>
-      <c r="K13" s="2" t="b">
+      <c r="K13" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" s="1" t="s">
         <v>50</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F14" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="G14" s="0" t="n">
+      <c r="F14" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="1" t="n">
         <f aca="false">F14*3</f>
         <v>9</v>
       </c>
-      <c r="H14" s="0" t="n">
+      <c r="H14" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="I14" s="0" t="n">
+      <c r="I14" s="1" t="n">
         <v>2.04</v>
       </c>
-      <c r="J14" s="0" t="n">
+      <c r="J14" s="1" t="n">
         <f aca="false">H14*I14</f>
         <v>24.48</v>
       </c>
-      <c r="K14" s="2" t="b">
+      <c r="K14" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" s="1" t="s">
         <v>53</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="F15" s="0" t="n">
+      <c r="F15" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="0" t="n">
+      <c r="G15" s="1" t="n">
         <f aca="false">F15*3</f>
         <v>6</v>
       </c>
-      <c r="H15" s="0" t="n">
+      <c r="H15" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="I15" s="0" t="n">
+      <c r="I15" s="1" t="n">
         <v>1.73</v>
       </c>
-      <c r="J15" s="0" t="n">
+      <c r="J15" s="1" t="n">
         <f aca="false">H15*I15</f>
         <v>13.84</v>
       </c>
-      <c r="K15" s="2" t="b">
+      <c r="K15" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F16" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="0" t="n">
+      <c r="F16" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="1" t="n">
         <f aca="false">F16*3</f>
         <v>3</v>
       </c>
-      <c r="H16" s="0" t="n">
+      <c r="H16" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I16" s="0" t="n">
+      <c r="I16" s="1" t="n">
         <v>3.06</v>
       </c>
-      <c r="J16" s="0" t="n">
+      <c r="J16" s="1" t="n">
         <f aca="false">H16*I16</f>
         <v>12.24</v>
       </c>
-      <c r="K16" s="2" t="b">
+      <c r="K16" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" s="1" t="s">
         <v>61</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F17" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" s="0" t="n">
+      <c r="F17" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="1" t="n">
         <f aca="false">F17*3</f>
         <v>3</v>
       </c>
-      <c r="H17" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="I17" s="0" t="n">
+      <c r="H17" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" s="1" t="n">
         <v>51.96</v>
       </c>
-      <c r="J17" s="0" t="n">
+      <c r="J17" s="1" t="n">
         <f aca="false">H17*I17</f>
         <v>155.88</v>
       </c>
-      <c r="K17" s="2" t="b">
+      <c r="K17" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D18" s="0" t="s">
+      <c r="D18" s="1" t="s">
         <v>65</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="F18" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="0" t="n">
+      <c r="F18" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="1" t="n">
         <f aca="false">F18*3</f>
         <v>3</v>
       </c>
-      <c r="H18" s="0" t="n">
+      <c r="H18" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I18" s="0" t="n">
+      <c r="I18" s="1" t="n">
         <v>38.1</v>
       </c>
-      <c r="J18" s="0" t="n">
+      <c r="J18" s="1" t="n">
         <f aca="false">H18*I18</f>
         <v>152.4</v>
       </c>
-      <c r="K18" s="2" t="b">
+      <c r="K18" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D19" s="0" t="s">
+      <c r="D19" s="1" t="s">
         <v>69</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="F19" s="0" t="n">
+      <c r="F19" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G19" s="0" t="n">
+      <c r="G19" s="1" t="n">
         <f aca="false">F19*3</f>
         <v>6</v>
       </c>
-      <c r="H19" s="0" t="n">
+      <c r="H19" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="I19" s="0" t="n">
+      <c r="I19" s="1" t="n">
         <v>33.21</v>
       </c>
-      <c r="J19" s="0" t="n">
+      <c r="J19" s="1" t="n">
         <f aca="false">H19*I19</f>
         <v>232.47</v>
       </c>
-      <c r="K19" s="2" t="b">
+      <c r="K19" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="D20" s="1" t="s">
         <v>73</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="F20" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" s="0" t="n">
+      <c r="F20" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="1" t="n">
         <f aca="false">F20*3</f>
         <v>3</v>
       </c>
-      <c r="H20" s="0" t="n">
+      <c r="H20" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I20" s="0" t="n">
+      <c r="I20" s="1" t="n">
         <v>48.9</v>
       </c>
-      <c r="J20" s="0" t="n">
+      <c r="J20" s="1" t="n">
         <f aca="false">H20*I20</f>
         <v>244.5</v>
       </c>
-      <c r="K20" s="2" t="b">
+      <c r="K20" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="G21" s="0" t="n">
+      <c r="C21" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="1" t="n">
         <f aca="false">F21*3</f>
-        <v>0</v>
-      </c>
-      <c r="J21" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I21" s="1" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="J21" s="1" t="n">
         <f aca="false">H21*I21</f>
-        <v>0</v>
-      </c>
-      <c r="K21" s="2" t="b">
+        <v>9.78</v>
+      </c>
+      <c r="K21" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="G22" s="0" t="n">
+      <c r="D22" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F22" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="1" t="n">
         <f aca="false">F22*3</f>
-        <v>0</v>
-      </c>
-      <c r="J22" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="H22" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I22" s="1" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="J22" s="1" t="n">
         <f aca="false">H22*I22</f>
-        <v>0</v>
-      </c>
-      <c r="K22" s="2" t="b">
+        <v>9.78</v>
+      </c>
+      <c r="K22" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="G23" s="0" t="n">
+      <c r="B23" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F23" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="1" t="n">
         <f aca="false">F23*3</f>
-        <v>0</v>
-      </c>
-      <c r="J23" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I23" s="1" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="J23" s="1" t="n">
         <f aca="false">H23*I23</f>
-        <v>0</v>
-      </c>
-      <c r="K23" s="2" t="b">
+        <v>23.22</v>
+      </c>
+      <c r="K23" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="G24" s="0" t="n">
+      <c r="B24" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>61300811121</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F24" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="1" t="n">
         <f aca="false">F24*3</f>
-        <v>0</v>
-      </c>
-      <c r="J24" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="H24" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I24" s="1" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="J24" s="1" t="n">
         <f aca="false">H24*I24</f>
-        <v>0</v>
-      </c>
-      <c r="K24" s="2" t="b">
+        <v>11.01</v>
+      </c>
+      <c r="K24" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="C25" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="D25" s="0" t="s">
-        <v>81</v>
+      <c r="B25" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="F25" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="0" t="n">
+        <v>90</v>
+      </c>
+      <c r="F25" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="1" t="n">
         <f aca="false">F25*3</f>
         <v>3</v>
       </c>
-      <c r="H25" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="I25" s="0" t="n">
+      <c r="H25" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I25" s="1" t="n">
         <v>1774.7</v>
       </c>
-      <c r="J25" s="0" t="n">
+      <c r="J25" s="1" t="n">
         <f aca="false">H25*I25</f>
         <v>5324.1</v>
       </c>
-      <c r="K25" s="2" t="b">
+      <c r="K25" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="0" t="s">
-        <v>83</v>
-      </c>
-      <c r="C26" s="0" t="s">
-        <v>84</v>
+      <c r="B26" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>92</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F26" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="0" t="n">
+        <v>94</v>
+      </c>
+      <c r="F26" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="1" t="n">
         <f aca="false">F26*3</f>
         <v>3</v>
       </c>
-      <c r="H26" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="I26" s="0" t="n">
+      <c r="H26" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" s="1" t="n">
         <v>19.05</v>
       </c>
-      <c r="J26" s="0" t="n">
+      <c r="J26" s="1" t="n">
         <f aca="false">H26*I26</f>
         <v>57.15</v>
       </c>
-      <c r="K26" s="2" t="b">
+      <c r="K26" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="F27" s="0" t="n">
+      <c r="B27" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>61300211121</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F27" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="G27" s="0" t="n">
+      <c r="G27" s="1" t="n">
         <f aca="false">F27*3</f>
         <v>12</v>
       </c>
-      <c r="J27" s="0" t="n">
+      <c r="H27" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="I27" s="1" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="J27" s="1" t="n">
         <f aca="false">H27*I27</f>
-        <v>0</v>
-      </c>
-      <c r="K27" s="2" t="b">
+        <v>14.64</v>
+      </c>
+      <c r="K27" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="F28" s="0" t="n">
+      <c r="B28" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="F28" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="G28" s="0" t="n">
+      <c r="G28" s="1" t="n">
         <f aca="false">F28*3</f>
         <v>12</v>
       </c>
-      <c r="J28" s="0" t="n">
+      <c r="H28" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="I28" s="1" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J28" s="1" t="n">
         <f aca="false">H28*I28</f>
-        <v>0</v>
-      </c>
-      <c r="K28" s="2" t="b">
+        <v>12.24</v>
+      </c>
+      <c r="K28" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="0" t="s">
-        <v>89</v>
+      <c r="B30" s="1" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="C31" s="0" t="n">
+      <c r="B31" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C31" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="F31" s="0" t="n">
+        <v>102</v>
+      </c>
+      <c r="F31" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="G31" s="0" t="n">
+      <c r="G31" s="1" t="n">
         <f aca="false">F31*3</f>
         <v>12</v>
       </c>
-      <c r="H31" s="0" t="n">
+      <c r="H31" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="I31" s="0" t="n">
+      <c r="I31" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J31" s="0" t="n">
+      <c r="J31" s="1" t="n">
         <f aca="false">H31*I31</f>
         <v>16.32</v>
       </c>
-      <c r="K31" s="2" t="b">
+      <c r="K31" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="C32" s="0" t="n">
+      <c r="B32" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C32" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F32" s="0" t="n">
+        <v>104</v>
+      </c>
+      <c r="F32" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G32" s="0" t="n">
+      <c r="G32" s="1" t="n">
         <f aca="false">F32*3</f>
         <v>6</v>
       </c>
-      <c r="H32" s="0" t="n">
+      <c r="H32" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="I32" s="0" t="n">
+      <c r="I32" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J32" s="0" t="n">
+      <c r="J32" s="1" t="n">
         <f aca="false">H32*I32</f>
         <v>8.16</v>
       </c>
-      <c r="K32" s="2" t="b">
+      <c r="K32" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="0" t="s">
-        <v>94</v>
-      </c>
-      <c r="C33" s="0" t="n">
+      <c r="B33" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C33" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="F33" s="0" t="n">
+        <v>106</v>
+      </c>
+      <c r="F33" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="G33" s="0" t="n">
+      <c r="G33" s="1" t="n">
         <f aca="false">F33*3</f>
         <v>42</v>
       </c>
-      <c r="H33" s="0" t="n">
+      <c r="H33" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="I33" s="0" t="n">
+      <c r="I33" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J33" s="0" t="n">
+      <c r="J33" s="1" t="n">
         <f aca="false">H33*I33</f>
         <v>51</v>
       </c>
-      <c r="K33" s="2" t="b">
+      <c r="K33" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="C34" s="0" t="n">
+      <c r="B34" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C34" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="F34" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="0" t="n">
+        <v>108</v>
+      </c>
+      <c r="F34" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="1" t="n">
         <f aca="false">F34*3</f>
         <v>3</v>
       </c>
-      <c r="H34" s="0" t="n">
+      <c r="H34" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I34" s="0" t="n">
+      <c r="I34" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J34" s="0" t="n">
+      <c r="J34" s="1" t="n">
         <f aca="false">H34*I34</f>
         <v>5.1</v>
       </c>
-      <c r="K34" s="2" t="b">
+      <c r="K34" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="0" t="s">
-        <v>98</v>
-      </c>
-      <c r="C35" s="0" t="n">
+      <c r="B35" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C35" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F35" s="0" t="n">
+        <v>110</v>
+      </c>
+      <c r="F35" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="G35" s="0" t="n">
+      <c r="G35" s="1" t="n">
         <f aca="false">F35*3</f>
         <v>45</v>
       </c>
-      <c r="H35" s="0" t="n">
+      <c r="H35" s="1" t="n">
         <v>55</v>
       </c>
-      <c r="I35" s="0" t="n">
+      <c r="I35" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J35" s="0" t="n">
+      <c r="J35" s="1" t="n">
         <f aca="false">H35*I35</f>
         <v>56.1</v>
       </c>
-      <c r="K35" s="2" t="b">
+      <c r="K35" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="0" t="s">
-        <v>100</v>
-      </c>
-      <c r="C36" s="0" t="n">
+      <c r="B36" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C36" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="F36" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" s="0" t="n">
+        <v>112</v>
+      </c>
+      <c r="F36" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="1" t="n">
         <f aca="false">F36*3</f>
         <v>3</v>
       </c>
-      <c r="H36" s="0" t="n">
+      <c r="H36" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I36" s="0" t="n">
+      <c r="I36" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J36" s="0" t="n">
+      <c r="J36" s="1" t="n">
         <f aca="false">H36*I36</f>
         <v>5.1</v>
       </c>
-      <c r="K36" s="2" t="b">
+      <c r="K36" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="C37" s="0" t="n">
+      <c r="B37" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C37" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="F37" s="0" t="n">
+        <v>114</v>
+      </c>
+      <c r="F37" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="G37" s="0" t="n">
+      <c r="G37" s="1" t="n">
         <f aca="false">F37*3</f>
         <v>39</v>
       </c>
-      <c r="H37" s="0" t="n">
+      <c r="H37" s="1" t="n">
         <v>44</v>
       </c>
-      <c r="I37" s="0" t="n">
+      <c r="I37" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J37" s="0" t="n">
+      <c r="J37" s="1" t="n">
         <f aca="false">H37*I37</f>
         <v>44.88</v>
       </c>
-      <c r="K37" s="2" t="b">
+      <c r="K37" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="C38" s="0" t="n">
+      <c r="B38" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C38" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="F38" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" s="0" t="n">
+        <v>116</v>
+      </c>
+      <c r="F38" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="1" t="n">
         <f aca="false">F38*3</f>
         <v>3</v>
       </c>
-      <c r="H38" s="0" t="n">
+      <c r="H38" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I38" s="0" t="n">
+      <c r="I38" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J38" s="0" t="n">
+      <c r="J38" s="1" t="n">
         <f aca="false">H38*I38</f>
         <v>5.1</v>
       </c>
-      <c r="K38" s="2" t="b">
+      <c r="K38" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="0" t="s">
-        <v>106</v>
-      </c>
-      <c r="C39" s="0" t="n">
+      <c r="B39" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C39" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="F39" s="0" t="n">
+        <v>118</v>
+      </c>
+      <c r="F39" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="G39" s="0" t="n">
+      <c r="G39" s="1" t="n">
         <f aca="false">F39*3</f>
         <v>12</v>
       </c>
-      <c r="H39" s="0" t="n">
+      <c r="H39" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="I39" s="0" t="n">
+      <c r="I39" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J39" s="0" t="n">
+      <c r="J39" s="1" t="n">
         <f aca="false">H39*I39</f>
         <v>15.3</v>
       </c>
-      <c r="K39" s="2" t="b">
+      <c r="K39" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B40" s="0" t="s">
-        <v>108</v>
-      </c>
-      <c r="C40" s="0" t="n">
+      <c r="B40" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C40" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="F40" s="0" t="n">
+        <v>120</v>
+      </c>
+      <c r="F40" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="G40" s="0" t="n">
+      <c r="G40" s="1" t="n">
         <f aca="false">F40*3</f>
         <v>12</v>
       </c>
-      <c r="H40" s="0" t="n">
+      <c r="H40" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="I40" s="0" t="n">
+      <c r="I40" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J40" s="0" t="n">
+      <c r="J40" s="1" t="n">
         <f aca="false">H40*I40</f>
         <v>15.3</v>
       </c>
-      <c r="K40" s="2" t="b">
+      <c r="K40" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B41" s="0" t="s">
-        <v>110</v>
-      </c>
-      <c r="C41" s="0" t="n">
+      <c r="B41" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C41" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="F41" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" s="0" t="n">
+        <v>122</v>
+      </c>
+      <c r="F41" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="1" t="n">
         <f aca="false">F41*3</f>
         <v>3</v>
       </c>
-      <c r="H41" s="0" t="n">
+      <c r="H41" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I41" s="0" t="n">
+      <c r="I41" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J41" s="0" t="n">
+      <c r="J41" s="1" t="n">
         <f aca="false">H41*I41</f>
         <v>5.1</v>
       </c>
-      <c r="K41" s="2" t="b">
+      <c r="K41" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B42" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="C42" s="0" t="n">
+      <c r="B42" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C42" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="F42" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" s="0" t="n">
+        <v>124</v>
+      </c>
+      <c r="F42" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="1" t="n">
         <f aca="false">F42*3</f>
         <v>3</v>
       </c>
-      <c r="H42" s="0" t="n">
+      <c r="H42" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I42" s="0" t="n">
+      <c r="I42" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J42" s="0" t="n">
+      <c r="J42" s="1" t="n">
         <f aca="false">H42*I42</f>
         <v>5.1</v>
       </c>
-      <c r="K42" s="2" t="b">
+      <c r="K42" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B43" s="0" t="s">
-        <v>114</v>
-      </c>
-      <c r="C43" s="0" t="n">
+      <c r="B43" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C43" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="F43" s="0" t="n">
+        <v>126</v>
+      </c>
+      <c r="F43" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="G43" s="0" t="n">
+      <c r="G43" s="1" t="n">
         <f aca="false">F43*3</f>
         <v>48</v>
       </c>
-      <c r="H43" s="0" t="n">
+      <c r="H43" s="1" t="n">
         <v>55</v>
       </c>
-      <c r="I43" s="0" t="n">
+      <c r="I43" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J43" s="0" t="n">
+      <c r="J43" s="1" t="n">
         <f aca="false">H43*I43</f>
         <v>56.1</v>
       </c>
-      <c r="K43" s="2" t="b">
+      <c r="K43" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="C44" s="0" t="n">
+      <c r="B44" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C44" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="F44" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" s="0" t="n">
+        <v>128</v>
+      </c>
+      <c r="F44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="1" t="n">
         <f aca="false">F44*3</f>
         <v>3</v>
       </c>
-      <c r="H44" s="0" t="n">
+      <c r="H44" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I44" s="0" t="n">
+      <c r="I44" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J44" s="0" t="n">
+      <c r="J44" s="1" t="n">
         <f aca="false">H44*I44</f>
         <v>5.1</v>
       </c>
-      <c r="K44" s="2" t="b">
+      <c r="K44" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B46" s="0" t="s">
-        <v>118</v>
+      <c r="B46" s="1" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B47" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="C47" s="0" t="n">
+      <c r="B47" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C47" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="F47" s="0" t="n">
+        <v>131</v>
+      </c>
+      <c r="F47" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G47" s="0" t="n">
+      <c r="G47" s="1" t="n">
         <f aca="false">F47*3</f>
         <v>6</v>
       </c>
-      <c r="H47" s="0" t="n">
+      <c r="H47" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="I47" s="0" t="n">
+      <c r="I47" s="1" t="n">
         <v>2.04</v>
       </c>
-      <c r="J47" s="0" t="n">
+      <c r="J47" s="1" t="n">
         <f aca="false">H47*I47</f>
         <v>16.32</v>
       </c>
-      <c r="K47" s="2" t="b">
+      <c r="K47" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B48" s="0" t="s">
-        <v>121</v>
-      </c>
-      <c r="C48" s="0" t="n">
+      <c r="B48" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C48" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="F48" s="0" t="n">
+        <v>133</v>
+      </c>
+      <c r="F48" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="G48" s="0" t="n">
+      <c r="G48" s="1" t="n">
         <f aca="false">F48*3</f>
         <v>63</v>
       </c>
-      <c r="H48" s="0" t="n">
+      <c r="H48" s="1" t="n">
         <v>70</v>
       </c>
-      <c r="I48" s="0" t="n">
+      <c r="I48" s="1" t="n">
         <v>0.82</v>
       </c>
-      <c r="J48" s="0" t="n">
+      <c r="J48" s="1" t="n">
         <f aca="false">H48*I48</f>
         <v>57.4</v>
       </c>
-      <c r="K48" s="2" t="b">
+      <c r="K48" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="0" t="s">
-        <v>123</v>
-      </c>
-      <c r="C49" s="0" t="n">
+      <c r="B49" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C49" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="F49" s="0" t="n">
+        <v>135</v>
+      </c>
+      <c r="F49" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="G49" s="0" t="n">
+      <c r="G49" s="1" t="n">
         <f aca="false">F49*3</f>
         <v>63</v>
       </c>
-      <c r="H49" s="0" t="n">
+      <c r="H49" s="1" t="n">
         <v>70</v>
       </c>
-      <c r="I49" s="0" t="n">
+      <c r="I49" s="1" t="n">
         <v>2.65</v>
       </c>
-      <c r="J49" s="0" t="n">
+      <c r="J49" s="1" t="n">
         <f aca="false">H49*I49</f>
         <v>185.5</v>
       </c>
-      <c r="K49" s="2" t="b">
+      <c r="K49" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B50" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="C50" s="0" t="n">
+      <c r="B50" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C50" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="F50" s="0" t="n">
+        <v>137</v>
+      </c>
+      <c r="F50" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="G50" s="0" t="n">
+      <c r="G50" s="1" t="n">
         <f aca="false">F50*3</f>
         <v>18</v>
       </c>
-      <c r="H50" s="0" t="n">
+      <c r="H50" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="I50" s="0" t="n">
+      <c r="I50" s="1" t="n">
         <v>0.82</v>
       </c>
-      <c r="J50" s="0" t="n">
+      <c r="J50" s="1" t="n">
         <f aca="false">H50*I50</f>
         <v>18.04</v>
       </c>
-      <c r="K50" s="2" t="b">
+      <c r="K50" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B51" s="0" t="s">
-        <v>127</v>
-      </c>
-      <c r="C51" s="0" t="n">
+      <c r="B51" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C51" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="F51" s="0" t="n">
+        <v>139</v>
+      </c>
+      <c r="F51" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G51" s="0" t="n">
+      <c r="G51" s="1" t="n">
         <f aca="false">F51*3</f>
         <v>6</v>
       </c>
-      <c r="H51" s="0" t="n">
+      <c r="H51" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="I51" s="0" t="n">
+      <c r="I51" s="1" t="n">
         <v>1.83</v>
       </c>
-      <c r="J51" s="0" t="n">
+      <c r="J51" s="1" t="n">
         <f aca="false">H51*I51</f>
         <v>14.64</v>
       </c>
-      <c r="K51" s="2" t="b">
+      <c r="K51" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B52" s="0" t="s">
-        <v>129</v>
-      </c>
-      <c r="C52" s="0" t="n">
+      <c r="B52" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C52" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="F52" s="0" t="n">
+        <v>141</v>
+      </c>
+      <c r="F52" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="G52" s="0" t="n">
+      <c r="G52" s="1" t="n">
         <f aca="false">F52*3</f>
         <v>36</v>
       </c>
-      <c r="H52" s="0" t="n">
+      <c r="H52" s="1" t="n">
         <v>42</v>
       </c>
-      <c r="I52" s="0" t="n">
+      <c r="I52" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J52" s="0" t="n">
+      <c r="J52" s="1" t="n">
         <f aca="false">H52*I52</f>
         <v>42.84</v>
       </c>
-      <c r="K52" s="2" t="b">
+      <c r="K52" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B53" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="C53" s="0" t="n">
+      <c r="B53" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C53" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="F53" s="0" t="n">
+        <v>143</v>
+      </c>
+      <c r="F53" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="G53" s="0" t="n">
+      <c r="G53" s="1" t="n">
         <f aca="false">F53*3</f>
         <v>12</v>
       </c>
-      <c r="H53" s="0" t="n">
+      <c r="H53" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="I53" s="0" t="n">
+      <c r="I53" s="1" t="n">
         <v>1.32</v>
       </c>
-      <c r="J53" s="0" t="n">
+      <c r="J53" s="1" t="n">
         <f aca="false">H53*I53</f>
         <v>19.8</v>
       </c>
-      <c r="K53" s="2" t="b">
+      <c r="K53" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B55" s="0" t="s">
-        <v>133</v>
-      </c>
-      <c r="C55" s="0" t="n">
+      <c r="B55" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C55" s="1" t="n">
         <v>1206</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="F55" s="0" t="n">
+        <v>145</v>
+      </c>
+      <c r="F55" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="G55" s="0" t="n">
+      <c r="G55" s="1" t="n">
         <f aca="false">F55*3</f>
         <v>24</v>
       </c>
-      <c r="H55" s="0" t="n">
+      <c r="H55" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="I55" s="0" t="n">
+      <c r="I55" s="1" t="n">
         <v>0.82</v>
       </c>
-      <c r="J55" s="0" t="n">
+      <c r="J55" s="1" t="n">
         <f aca="false">H55*I55</f>
         <v>22.96</v>
       </c>
-      <c r="K55" s="2" t="b">
+      <c r="K55" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B56" s="0" t="s">
-        <v>135</v>
-      </c>
-      <c r="C56" s="0" t="n">
+      <c r="B56" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C56" s="1" t="n">
         <v>1206</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="F56" s="0" t="n">
+        <v>147</v>
+      </c>
+      <c r="F56" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="G56" s="0" t="n">
+      <c r="G56" s="1" t="n">
         <f aca="false">F56*3</f>
         <v>24</v>
       </c>
-      <c r="H56" s="0" t="n">
+      <c r="H56" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="I56" s="0" t="n">
+      <c r="I56" s="1" t="n">
         <v>0.92</v>
       </c>
-      <c r="J56" s="0" t="n">
+      <c r="J56" s="1" t="n">
         <f aca="false">H56*I56</f>
         <v>25.76</v>
       </c>
-      <c r="K56" s="2" t="b">
+      <c r="K56" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B57" s="0" t="s">
-        <v>137</v>
-      </c>
-      <c r="C57" s="0" t="n">
+      <c r="B57" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C57" s="1" t="n">
         <v>1206</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="F57" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G57" s="0" t="n">
+        <v>149</v>
+      </c>
+      <c r="F57" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="1" t="n">
         <f aca="false">F57*3</f>
         <v>3</v>
       </c>
-      <c r="H57" s="0" t="n">
+      <c r="H57" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I57" s="0" t="n">
+      <c r="I57" s="1" t="n">
         <v>4.08</v>
       </c>
-      <c r="J57" s="0" t="n">
+      <c r="J57" s="1" t="n">
         <f aca="false">H57*I57</f>
         <v>20.4</v>
       </c>
-      <c r="K57" s="2" t="b">
+      <c r="K57" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B59" s="0" t="s">
-        <v>139</v>
-      </c>
-      <c r="C59" s="0" t="n">
+      <c r="B59" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C59" s="1" t="n">
         <v>1210</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="F59" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G59" s="0" t="n">
+        <v>151</v>
+      </c>
+      <c r="F59" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="1" t="n">
         <f aca="false">F59*3</f>
         <v>3</v>
       </c>
-      <c r="H59" s="0" t="n">
+      <c r="H59" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I59" s="0" t="n">
+      <c r="I59" s="1" t="n">
         <v>16.61</v>
       </c>
-      <c r="J59" s="0" t="n">
+      <c r="J59" s="1" t="n">
         <f aca="false">H59*I59</f>
         <v>66.44</v>
       </c>
-      <c r="K59" s="2" t="b">
+      <c r="K59" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B61" s="0" t="s">
-        <v>141</v>
+      <c r="B61" s="1" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B62" s="0" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C62" s="0" t="n">
+      <c r="B62" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="C62" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="F62" s="0" t="n">
+        <v>154</v>
+      </c>
+      <c r="F62" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G62" s="0" t="n">
+      <c r="G62" s="1" t="n">
         <f aca="false">F62*3</f>
         <v>6</v>
       </c>
-      <c r="H62" s="0" t="n">
+      <c r="H62" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="I62" s="0" t="n">
+      <c r="I62" s="1" t="n">
         <v>1.73</v>
       </c>
-      <c r="J62" s="0" t="n">
+      <c r="J62" s="1" t="n">
         <f aca="false">H62*I62</f>
         <v>13.84</v>
       </c>
-      <c r="K62" s="2" t="b">
+      <c r="K62" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B63" s="0" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="C63" s="0" t="n">
+      <c r="B63" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C63" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="F63" s="0" t="n">
+        <v>156</v>
+      </c>
+      <c r="F63" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G63" s="0" t="n">
+      <c r="G63" s="1" t="n">
         <f aca="false">F63*3</f>
         <v>6</v>
       </c>
-      <c r="H63" s="0" t="n">
+      <c r="H63" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="I63" s="0" t="n">
+      <c r="I63" s="1" t="n">
         <v>2.45</v>
       </c>
-      <c r="J63" s="0" t="n">
+      <c r="J63" s="1" t="n">
         <f aca="false">H63*I63</f>
         <v>19.6</v>
       </c>
-      <c r="K63" s="2" t="b">
+      <c r="K63" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B64" s="0" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="C64" s="0" t="n">
+      <c r="B64" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C64" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="F64" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G64" s="0" t="n">
+        <v>158</v>
+      </c>
+      <c r="F64" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="1" t="n">
         <f aca="false">F64*3</f>
         <v>3</v>
       </c>
-      <c r="H64" s="0" t="n">
+      <c r="H64" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I64" s="0" t="n">
+      <c r="I64" s="1" t="n">
         <v>1.73</v>
       </c>
-      <c r="J64" s="0" t="n">
+      <c r="J64" s="1" t="n">
         <f aca="false">H64*I64</f>
         <v>8.65</v>
       </c>
-      <c r="K64" s="2" t="b">
+      <c r="K64" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I66" s="0" t="s">
-        <v>145</v>
-      </c>
-      <c r="J66" s="0" t="n">
+      <c r="I66" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="J66" s="1" t="n">
         <f aca="false">SUM(J3:J65)</f>
-        <v>9828.29</v>
-      </c>
-      <c r="K66" s="0" t="s">
-        <v>146</v>
+        <v>9908.96</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
feat: add buttons and VGA transceiver to shopping list
We had forgotten to add these elements to the list. Now the list
consists of 211 components per PCB.

The Bill of Materials (BoM) is telling us that we have footprints for
203 components per PCB.
We get 211 components per PCB, because 8 components do not have a
footprint on the board. These components are:

LCD Display (1x)
LCD Breakout 45pin (1x)
LCD Breakout 6pin (1x)
15V Power Supply (1x)
Jumper Cap (4x)
</commit_message>
<xml_diff>
--- a/Handleliste-hardware.xlsx
+++ b/Handleliste-hardware.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="173">
   <si>
     <t xml:space="preserve">Komponent</t>
   </si>
@@ -154,7 +154,7 @@
     <t xml:space="preserve">-</t>
   </si>
   <si>
-    <t xml:space="preserve">USB-A</t>
+    <t xml:space="preserve">USB-A port</t>
   </si>
   <si>
     <t xml:space="preserve">On Shore Technology Inc.</t>
@@ -166,6 +166,42 @@
     <t xml:space="preserve">https://www.digikey.no/no/products/detail/on-shore-technology-inc/USB-A1HSW6/2677750 </t>
   </si>
   <si>
+    <t xml:space="preserve">Undo/Reset Button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C&amp;K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KS11R21CQD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/en/products/detail/c-k/KS11R21CQD/332668</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cheap Button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E-Switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PS1024ABLK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/en/products/detail/e-switch/PS1024ABLK/81742</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VGA Transceiver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texas Instruments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SN74ALVC245PWR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/en/products/detail/texas-instruments/SN74ALVC245PWR/381176?s=N4IgTCBcDaIMoDkDsAWAggGQGoGEwoFYAFAdQCUQBdAXyA</t>
+  </si>
+  <si>
     <t xml:space="preserve">LED (Grønn)</t>
   </si>
   <si>
@@ -226,9 +262,6 @@
     <t xml:space="preserve">Nedtransformator (Power Supply)</t>
   </si>
   <si>
-    <t xml:space="preserve">Texas Instruments</t>
-  </si>
-  <si>
     <t xml:space="preserve">TPS54294PWP</t>
   </si>
   <si>
@@ -497,6 +530,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.digikey.no/no/products/detail/murata-electronics/LQM21PN3R3MGRD/4359175 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antall komponenter per PCB:</t>
   </si>
   <si>
     <t xml:space="preserve">tot sum</t>
@@ -892,7 +928,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:K1048576"/>
+  <dimension ref="A2:K68"/>
   <sheetFormatPr defaultColWidth="8.55859375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.11"/>
@@ -1281,9 +1317,34 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>2</v>
+      </c>
       <c r="G13" s="1" t="n">
         <f aca="false">F13*3</f>
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="H13" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="I13" s="1" t="n">
+        <v>28.93</v>
+      </c>
+      <c r="J13" s="1" t="n">
+        <f aca="false">H13*I13</f>
+        <v>231.44</v>
       </c>
       <c r="K13" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1292,33 +1353,33 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>55</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G14" s="1" t="n">
         <f aca="false">F14*3</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H14" s="1" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>2.04</v>
+        <v>17.42</v>
       </c>
       <c r="J14" s="1" t="n">
         <f aca="false">H14*I14</f>
-        <v>24.48</v>
+        <v>243.88</v>
       </c>
       <c r="K14" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1327,16 +1388,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>54</v>
+        <v>58</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="F15" s="1" t="n">
         <v>2</v>
@@ -1349,11 +1410,11 @@
         <v>8</v>
       </c>
       <c r="I15" s="1" t="n">
-        <v>1.73</v>
+        <v>7.64</v>
       </c>
       <c r="J15" s="1" t="n">
         <f aca="false">H15*I15</f>
-        <v>13.84</v>
+        <v>61.12</v>
       </c>
       <c r="K15" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1362,33 +1423,33 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G16" s="1" t="n">
         <f aca="false">F16*3</f>
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H16" s="1" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I16" s="1" t="n">
-        <v>3.06</v>
+        <v>2.04</v>
       </c>
       <c r="J16" s="1" t="n">
         <f aca="false">H16*I16</f>
-        <v>12.24</v>
+        <v>24.48</v>
       </c>
       <c r="K16" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1397,33 +1458,33 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G17" s="1" t="n">
         <f aca="false">F17*3</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H17" s="1" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I17" s="1" t="n">
-        <v>51.96</v>
+        <v>1.73</v>
       </c>
       <c r="J17" s="1" t="n">
         <f aca="false">H17*I17</f>
-        <v>155.88</v>
+        <v>13.84</v>
       </c>
       <c r="K17" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1432,16 +1493,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="F18" s="1" t="n">
         <v>1</v>
@@ -1454,11 +1515,11 @@
         <v>4</v>
       </c>
       <c r="I18" s="1" t="n">
-        <v>38.1</v>
+        <v>3.06</v>
       </c>
       <c r="J18" s="1" t="n">
         <f aca="false">H18*I18</f>
-        <v>152.4</v>
+        <v>12.24</v>
       </c>
       <c r="K18" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1467,33 +1528,33 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G19" s="1" t="n">
         <f aca="false">F19*3</f>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H19" s="1" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I19" s="1" t="n">
-        <v>33.21</v>
+        <v>51.96</v>
       </c>
       <c r="J19" s="1" t="n">
         <f aca="false">H19*I19</f>
-        <v>232.47</v>
+        <v>155.88</v>
       </c>
       <c r="K19" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1502,16 +1563,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>1</v>
@@ -1521,14 +1582,14 @@
         <v>3</v>
       </c>
       <c r="H20" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I20" s="1" t="n">
-        <v>48.9</v>
+        <v>38.1</v>
       </c>
       <c r="J20" s="1" t="n">
         <f aca="false">H20*I20</f>
-        <v>244.5</v>
+        <v>152.4</v>
       </c>
       <c r="K20" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1537,33 +1598,33 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>81</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" s="1" t="n">
         <f aca="false">F21*3</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H21" s="1" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I21" s="1" t="n">
-        <v>3.26</v>
+        <v>33.21</v>
       </c>
       <c r="J21" s="1" t="n">
         <f aca="false">H21*I21</f>
-        <v>9.78</v>
+        <v>232.47</v>
       </c>
       <c r="K21" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1572,16 +1633,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>85</v>
       </c>
       <c r="F22" s="1" t="n">
         <v>1</v>
@@ -1591,14 +1652,14 @@
         <v>3</v>
       </c>
       <c r="H22" s="1" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I22" s="1" t="n">
-        <v>3.26</v>
+        <v>48.9</v>
       </c>
       <c r="J22" s="1" t="n">
         <f aca="false">H22*I22</f>
-        <v>9.78</v>
+        <v>244.5</v>
       </c>
       <c r="K22" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1607,16 +1668,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="F23" s="1" t="n">
         <v>1</v>
@@ -1629,11 +1690,11 @@
         <v>3</v>
       </c>
       <c r="I23" s="1" t="n">
-        <v>7.74</v>
+        <v>3.26</v>
       </c>
       <c r="J23" s="1" t="n">
         <f aca="false">H23*I23</f>
-        <v>23.22</v>
+        <v>9.78</v>
       </c>
       <c r="K23" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1642,16 +1703,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="1" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D24" s="1" t="n">
-        <v>61300811121</v>
+        <v>87</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F24" s="1" t="n">
         <v>1</v>
@@ -1664,11 +1725,11 @@
         <v>3</v>
       </c>
       <c r="I24" s="1" t="n">
-        <v>3.67</v>
+        <v>3.26</v>
       </c>
       <c r="J24" s="1" t="n">
         <f aca="false">H24*I24</f>
-        <v>11.01</v>
+        <v>9.78</v>
       </c>
       <c r="K24" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1677,16 +1738,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>94</v>
       </c>
       <c r="F25" s="1" t="n">
         <v>1</v>
@@ -1699,11 +1760,11 @@
         <v>3</v>
       </c>
       <c r="I25" s="1" t="n">
-        <v>1774.7</v>
+        <v>7.74</v>
       </c>
       <c r="J25" s="1" t="n">
         <f aca="false">H25*I25</f>
-        <v>5324.1</v>
+        <v>23.22</v>
       </c>
       <c r="K25" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1712,16 +1773,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>61300811121</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="F26" s="1" t="n">
         <v>1</v>
@@ -1734,11 +1795,11 @@
         <v>3</v>
       </c>
       <c r="I26" s="1" t="n">
-        <v>19.05</v>
+        <v>3.67</v>
       </c>
       <c r="J26" s="1" t="n">
         <f aca="false">H26*I26</f>
-        <v>57.15</v>
+        <v>11.01</v>
       </c>
       <c r="K26" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1747,33 +1808,33 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="1" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D27" s="1" t="n">
-        <v>61300211121</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>96</v>
+        <v>99</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>101</v>
       </c>
       <c r="F27" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G27" s="1" t="n">
         <f aca="false">F27*3</f>
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H27" s="1" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I27" s="1" t="n">
-        <v>1.22</v>
+        <v>1774.7</v>
       </c>
       <c r="J27" s="1" t="n">
         <f aca="false">H27*I27</f>
-        <v>14.64</v>
+        <v>5324.1</v>
       </c>
       <c r="K27" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1782,134 +1843,140 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="1" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>105</v>
       </c>
       <c r="F28" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G28" s="1" t="n">
         <f aca="false">F28*3</f>
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H28" s="1" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I28" s="1" t="n">
-        <v>1.02</v>
+        <v>19.05</v>
       </c>
       <c r="J28" s="1" t="n">
         <f aca="false">H28*I28</f>
-        <v>12.24</v>
+        <v>57.15</v>
       </c>
       <c r="K28" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>61300211121</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F29" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="G29" s="1" t="n">
+        <f aca="false">F29*3</f>
+        <v>12</v>
+      </c>
+      <c r="H29" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="I29" s="1" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="J29" s="1" t="n">
+        <f aca="false">H29*I29</f>
+        <v>14.64</v>
+      </c>
+      <c r="K29" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C31" s="1" t="n">
-        <v>805</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="F31" s="1" t="n">
+        <v>108</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F30" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="G31" s="1" t="n">
-        <f aca="false">F31*3</f>
+      <c r="G30" s="1" t="n">
+        <f aca="false">F30*3</f>
         <v>12</v>
       </c>
-      <c r="H31" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="I31" s="1" t="n">
+      <c r="H30" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="I30" s="1" t="n">
         <v>1.02</v>
       </c>
-      <c r="J31" s="1" t="n">
-        <f aca="false">H31*I31</f>
-        <v>16.32</v>
-      </c>
-      <c r="K31" s="1" t="b">
+      <c r="J30" s="1" t="n">
+        <f aca="false">H30*I30</f>
+        <v>12.24</v>
+      </c>
+      <c r="K30" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C32" s="1" t="n">
-        <v>805</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="F32" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G32" s="1" t="n">
-        <f aca="false">F32*3</f>
-        <v>6</v>
-      </c>
-      <c r="H32" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="I32" s="1" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="J32" s="1" t="n">
-        <f aca="false">H32*I32</f>
-        <v>8.16</v>
-      </c>
-      <c r="K32" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>111</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="1" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="C33" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="F33" s="1" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="G33" s="1" t="n">
         <f aca="false">F33*3</f>
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="H33" s="1" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="I33" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J33" s="1" t="n">
         <f aca="false">H33*I33</f>
-        <v>51</v>
+        <v>16.32</v>
       </c>
       <c r="K33" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1918,30 +1985,30 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="1" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="C34" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="F34" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G34" s="1" t="n">
         <f aca="false">F34*3</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H34" s="1" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I34" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J34" s="1" t="n">
         <f aca="false">H34*I34</f>
-        <v>5.1</v>
+        <v>8.16</v>
       </c>
       <c r="K34" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1950,30 +2017,30 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="1" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="C35" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="F35" s="1" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G35" s="1" t="n">
         <f aca="false">F35*3</f>
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="H35" s="1" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="I35" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J35" s="1" t="n">
         <f aca="false">H35*I35</f>
-        <v>56.1</v>
+        <v>51</v>
       </c>
       <c r="K35" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1982,13 +2049,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="1" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="C36" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="F36" s="1" t="n">
         <v>1</v>
@@ -2014,30 +2081,30 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="1" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="C37" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="F37" s="1" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G37" s="1" t="n">
         <f aca="false">F37*3</f>
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="H37" s="1" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="I37" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J37" s="1" t="n">
         <f aca="false">H37*I37</f>
-        <v>44.88</v>
+        <v>56.1</v>
       </c>
       <c r="K37" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -2046,13 +2113,13 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="1" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="C38" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="F38" s="1" t="n">
         <v>1</v>
@@ -2078,30 +2145,30 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="1" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="C39" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="F39" s="1" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="G39" s="1" t="n">
         <f aca="false">F39*3</f>
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="H39" s="1" t="n">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="I39" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J39" s="1" t="n">
         <f aca="false">H39*I39</f>
-        <v>15.3</v>
+        <v>44.88</v>
       </c>
       <c r="K39" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -2110,30 +2177,30 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="1" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C40" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="F40" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G40" s="1" t="n">
         <f aca="false">F40*3</f>
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H40" s="1" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="I40" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J40" s="1" t="n">
         <f aca="false">H40*I40</f>
-        <v>15.3</v>
+        <v>5.1</v>
       </c>
       <c r="K40" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -2142,30 +2209,30 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="1" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="C41" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="F41" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G41" s="1" t="n">
         <f aca="false">F41*3</f>
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H41" s="1" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="I41" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J41" s="1" t="n">
         <f aca="false">H41*I41</f>
-        <v>5.1</v>
+        <v>15.3</v>
       </c>
       <c r="K41" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -2174,30 +2241,30 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="1" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="C42" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="F42" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G42" s="1" t="n">
         <f aca="false">F42*3</f>
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H42" s="1" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="I42" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J42" s="1" t="n">
         <f aca="false">H42*I42</f>
-        <v>5.1</v>
+        <v>15.3</v>
       </c>
       <c r="K42" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -2206,30 +2273,30 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="1" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="C43" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="F43" s="1" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G43" s="1" t="n">
         <f aca="false">F43*3</f>
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="H43" s="1" t="n">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="I43" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J43" s="1" t="n">
         <f aca="false">H43*I43</f>
-        <v>56.1</v>
+        <v>5.1</v>
       </c>
       <c r="K43" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -2238,13 +2305,13 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="1" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C44" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="F44" s="1" t="n">
         <v>1</v>
@@ -2268,101 +2335,101 @@
         <v>0</v>
       </c>
     </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B45" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C45" s="1" t="n">
+        <v>805</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="F45" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="G45" s="1" t="n">
+        <f aca="false">F45*3</f>
+        <v>48</v>
+      </c>
+      <c r="H45" s="1" t="n">
+        <v>55</v>
+      </c>
+      <c r="I45" s="1" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J45" s="1" t="n">
+        <f aca="false">H45*I45</f>
+        <v>56.1</v>
+      </c>
+      <c r="K45" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B47" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="C47" s="1" t="n">
+        <v>138</v>
+      </c>
+      <c r="C46" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E47" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="F47" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G47" s="1" t="n">
-        <f aca="false">F47*3</f>
-        <v>6</v>
-      </c>
-      <c r="H47" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="I47" s="1" t="n">
-        <v>2.04</v>
-      </c>
-      <c r="J47" s="1" t="n">
-        <f aca="false">H47*I47</f>
-        <v>16.32</v>
-      </c>
-      <c r="K47" s="1" t="b">
+      <c r="E46" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="F46" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="1" t="n">
+        <f aca="false">F46*3</f>
+        <v>3</v>
+      </c>
+      <c r="H46" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="I46" s="1" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J46" s="1" t="n">
+        <f aca="false">H46*I46</f>
+        <v>5.1</v>
+      </c>
+      <c r="K46" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="C48" s="1" t="n">
-        <v>805</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="F48" s="1" t="n">
-        <v>21</v>
-      </c>
-      <c r="G48" s="1" t="n">
-        <f aca="false">F48*3</f>
-        <v>63</v>
-      </c>
-      <c r="H48" s="1" t="n">
-        <v>70</v>
-      </c>
-      <c r="I48" s="1" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="J48" s="1" t="n">
-        <f aca="false">H48*I48</f>
-        <v>57.4</v>
-      </c>
-      <c r="K48" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>140</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="1" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C49" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="F49" s="1" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="G49" s="1" t="n">
         <f aca="false">F49*3</f>
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="H49" s="1" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="I49" s="1" t="n">
-        <v>2.65</v>
+        <v>2.04</v>
       </c>
       <c r="J49" s="1" t="n">
         <f aca="false">H49*I49</f>
-        <v>185.5</v>
+        <v>16.32</v>
       </c>
       <c r="K49" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -2371,30 +2438,30 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="1" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C50" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="F50" s="1" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="G50" s="1" t="n">
         <f aca="false">F50*3</f>
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="H50" s="1" t="n">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="I50" s="1" t="n">
         <v>0.82</v>
       </c>
       <c r="J50" s="1" t="n">
         <f aca="false">H50*I50</f>
-        <v>18.04</v>
+        <v>57.4</v>
       </c>
       <c r="K50" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -2403,30 +2470,30 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="1" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="C51" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="F51" s="1" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="G51" s="1" t="n">
         <f aca="false">F51*3</f>
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="H51" s="1" t="n">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="I51" s="1" t="n">
-        <v>1.83</v>
+        <v>2.65</v>
       </c>
       <c r="J51" s="1" t="n">
         <f aca="false">H51*I51</f>
-        <v>14.64</v>
+        <v>185.5</v>
       </c>
       <c r="K51" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -2435,30 +2502,30 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="1" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="C52" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="F52" s="1" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="G52" s="1" t="n">
         <f aca="false">F52*3</f>
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="H52" s="1" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="I52" s="1" t="n">
-        <v>1.02</v>
+        <v>0.82</v>
       </c>
       <c r="J52" s="1" t="n">
         <f aca="false">H52*I52</f>
-        <v>42.84</v>
+        <v>18.04</v>
       </c>
       <c r="K52" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -2467,141 +2534,173 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="1" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C53" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="F53" s="1" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G53" s="1" t="n">
         <f aca="false">F53*3</f>
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H53" s="1" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="I53" s="1" t="n">
-        <v>1.32</v>
+        <v>1.83</v>
       </c>
       <c r="J53" s="1" t="n">
         <f aca="false">H53*I53</f>
-        <v>19.8</v>
+        <v>14.64</v>
       </c>
       <c r="K53" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B54" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C54" s="1" t="n">
+        <v>805</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="F54" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="G54" s="1" t="n">
+        <f aca="false">F54*3</f>
+        <v>36</v>
+      </c>
+      <c r="H54" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="I54" s="1" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J54" s="1" t="n">
+        <f aca="false">H54*I54</f>
+        <v>42.84</v>
+      </c>
+      <c r="K54" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="1" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="C55" s="1" t="n">
-        <v>1206</v>
+        <v>805</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="F55" s="1" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G55" s="1" t="n">
         <f aca="false">F55*3</f>
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H55" s="1" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="I55" s="1" t="n">
-        <v>0.82</v>
+        <v>1.32</v>
       </c>
       <c r="J55" s="1" t="n">
         <f aca="false">H55*I55</f>
-        <v>22.96</v>
+        <v>19.8</v>
       </c>
       <c r="K55" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B56" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="C56" s="1" t="n">
-        <v>1206</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="F56" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="G56" s="1" t="n">
-        <f aca="false">F56*3</f>
-        <v>24</v>
-      </c>
-      <c r="H56" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="I56" s="1" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="J56" s="1" t="n">
-        <f aca="false">H56*I56</f>
-        <v>25.76</v>
-      </c>
-      <c r="K56" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="1" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C57" s="1" t="n">
         <v>1206</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="F57" s="1" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G57" s="1" t="n">
         <f aca="false">F57*3</f>
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="H57" s="1" t="n">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="I57" s="1" t="n">
-        <v>4.08</v>
+        <v>0.82</v>
       </c>
       <c r="J57" s="1" t="n">
         <f aca="false">H57*I57</f>
-        <v>20.4</v>
+        <v>22.96</v>
       </c>
       <c r="K57" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B58" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C58" s="1" t="n">
+        <v>1206</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="F58" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="G58" s="1" t="n">
+        <f aca="false">F58*3</f>
+        <v>24</v>
+      </c>
+      <c r="H58" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="I58" s="1" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J58" s="1" t="n">
+        <f aca="false">H58*I58</f>
+        <v>25.76</v>
+      </c>
+      <c r="K58" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B59" s="1" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="C59" s="1" t="n">
-        <v>1210</v>
+        <v>1206</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="F59" s="1" t="n">
         <v>1</v>
@@ -2611,14 +2710,14 @@
         <v>3</v>
       </c>
       <c r="H59" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I59" s="1" t="n">
-        <v>16.61</v>
+        <v>4.08</v>
       </c>
       <c r="J59" s="1" t="n">
         <f aca="false">H59*I59</f>
-        <v>66.44</v>
+        <v>20.4</v>
       </c>
       <c r="K59" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -2627,118 +2726,156 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B61" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B62" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="C62" s="1" t="n">
-        <v>805</v>
-      </c>
-      <c r="E62" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="F62" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G62" s="1" t="n">
-        <f aca="false">F62*3</f>
-        <v>6</v>
-      </c>
-      <c r="H62" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="I62" s="1" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="J62" s="1" t="n">
-        <f aca="false">H62*I62</f>
-        <v>13.84</v>
-      </c>
-      <c r="K62" s="1" t="b">
+        <v>161</v>
+      </c>
+      <c r="C61" s="1" t="n">
+        <v>1210</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F61" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="1" t="n">
+        <f aca="false">F61*3</f>
+        <v>3</v>
+      </c>
+      <c r="H61" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="I61" s="1" t="n">
+        <v>16.61</v>
+      </c>
+      <c r="J61" s="1" t="n">
+        <f aca="false">H61*I61</f>
+        <v>66.44</v>
+      </c>
+      <c r="K61" s="1" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B63" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="C63" s="1" t="n">
-        <v>805</v>
-      </c>
-      <c r="E63" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="F63" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G63" s="1" t="n">
-        <f aca="false">F63*3</f>
-        <v>6</v>
-      </c>
-      <c r="H63" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="I63" s="1" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="J63" s="1" t="n">
-        <f aca="false">H63*I63</f>
-        <v>19.6</v>
-      </c>
-      <c r="K63" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>163</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="1" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C64" s="1" t="n">
         <v>805</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="F64" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G64" s="1" t="n">
         <f aca="false">F64*3</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H64" s="1" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I64" s="1" t="n">
         <v>1.73</v>
       </c>
       <c r="J64" s="1" t="n">
         <f aca="false">H64*I64</f>
+        <v>13.84</v>
+      </c>
+      <c r="K64" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B65" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C65" s="1" t="n">
+        <v>805</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F65" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G65" s="1" t="n">
+        <f aca="false">F65*3</f>
+        <v>6</v>
+      </c>
+      <c r="H65" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="I65" s="1" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="J65" s="1" t="n">
+        <f aca="false">H65*I65</f>
+        <v>19.6</v>
+      </c>
+      <c r="K65" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B66" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C66" s="1" t="n">
+        <v>805</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="F66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="1" t="n">
+        <f aca="false">F66*3</f>
+        <v>3</v>
+      </c>
+      <c r="H66" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="I66" s="1" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="J66" s="1" t="n">
+        <f aca="false">H66*I66</f>
         <v>8.65</v>
       </c>
-      <c r="K64" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I66" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="J66" s="1" t="n">
-        <f aca="false">SUM(J3:J65)</f>
-        <v>9908.96</v>
-      </c>
-      <c r="K66" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+      <c r="K66" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E68" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F68" s="1" t="n">
+        <f aca="false">SUM(F3:F66)</f>
+        <v>211</v>
+      </c>
+      <c r="I68" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="J68" s="1" t="n">
+        <f aca="false">SUM(J3:J67)</f>
+        <v>10445.4</v>
+      </c>
+      <c r="K68" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E3" r:id="rId1" display="https://www.digikey.no/no/products/detail/stmicroelectronics/STM32U5G7VJT6Q/21700656"/>
@@ -2751,43 +2888,43 @@
     <hyperlink ref="E10" r:id="rId8" display="https://www.digikey.no/no/products/detail/phihong-usa/PSA15R-150P6-R/5247157"/>
     <hyperlink ref="E11" r:id="rId9" display="https://www.digikey.no/no/products/detail/stmicroelectronics/STLINK-V3MINIE/16284301 "/>
     <hyperlink ref="E12" r:id="rId10" display="https://www.digikey.no/no/products/detail/on-shore-technology-inc/USB-A1HSW6/2677750 "/>
-    <hyperlink ref="E14" r:id="rId11" display="https://www.digikey.no/no/products/detail/liteon/LTST-C193KGKT-5A/2356242 "/>
-    <hyperlink ref="E15" r:id="rId12" display="https://www.digikey.no/no/products/detail/liteon/LTST-C193KRKT-5A/2356244 "/>
-    <hyperlink ref="E16" r:id="rId13" display="https://www.digikey.no/no/products/detail/murata-electronics/XRCGB48M000F4M00R0/2368388 "/>
-    <hyperlink ref="E17" r:id="rId14" display="https://www.digikey.no/no/products/detail/connor-winfield/CWX813-100-0M/695541 "/>
-    <hyperlink ref="E18" r:id="rId15" display="https://www.digikey.no/no/products/detail/gigadevice-semiconductor-hk-limited/GD25F128FS2GR/20531633 "/>
-    <hyperlink ref="E19" r:id="rId16" display="https://www.digikey.no/no/products/detail/texas-instruments/TPS54294PWP/2812688 "/>
-    <hyperlink ref="E20" r:id="rId17" display="https://www.digikey.no/no/products/detail/issi-integrated-silicon-solution-inc/IS66WVH16M8DBLL-100B1LI/6202025 "/>
-    <hyperlink ref="E25" r:id="rId18" display="https://www.digikey.no/no/products/detail/amd/XC7A100T-2FTG256I/3925791?s=N4IgTCBcDaIBoGEDsBBAjABgwFQLRgDFsBxMAVgDYBJEAXQF8g "/>
-    <hyperlink ref="E26" r:id="rId19" display="https://www.digikey.no/en/products/detail/amphenol-cs-commercial-products/L77HDE15SD1CH4RHNVGA/25816614 "/>
-    <hyperlink ref="E31" r:id="rId20" display="https://www.digikey.no/no/products/detail/stackpole-electronics-inc/RMCF0805JT47R0/1757848 "/>
-    <hyperlink ref="E32" r:id="rId21" display="https://www.digikey.no/no/products/detail/panasonic-electronic-components/ERA-6AEB101V/1465724 "/>
-    <hyperlink ref="E33" r:id="rId22" display="https://www.digikey.no/no/products/detail/vishay-dale/CRCW0805270RFKEAC/7922379  "/>
-    <hyperlink ref="E34" r:id="rId23" display="https://www.digikey.no/no/products/detail/stackpole-electronics-inc/RMCF0805FT330R/1760484"/>
-    <hyperlink ref="E35" r:id="rId24" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-07536RL/728026 "/>
-    <hyperlink ref="E36" r:id="rId25" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-072K4L/727690"/>
-    <hyperlink ref="E37" r:id="rId26" display="https://www.digikey.no/no/products/detail/vishay-dale/CRCW08054K70FKEAC/7928553 "/>
-    <hyperlink ref="E38" r:id="rId27" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-076K81L/728068 "/>
-    <hyperlink ref="E39" r:id="rId28" display="https://www.digikey.no/no/products/detail/susumu/RR1220P-103-D/432315 "/>
-    <hyperlink ref="E40" r:id="rId29" display="https://www.digikey.no/no/products/detail/stackpole-electronics-inc/RMCF0805FT22K1/1760211 "/>
-    <hyperlink ref="E41" r:id="rId30" display="https://www.digikey.no/no/products/detail/vishay-dale/CRCW080530K1FKEA/1175804 "/>
-    <hyperlink ref="E42" r:id="rId31" display="https://www.digikey.no/no/products/detail/panasonic-electronic-components/ERA-6AEB7322V/2025832 "/>
-    <hyperlink ref="E43" r:id="rId32" display="https://www.digikey.no/no/products/detail/susumu/RG2012P-104-B-T5/1240656 "/>
-    <hyperlink ref="E44" r:id="rId33" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-07124KL/727580 "/>
-    <hyperlink ref="E47" r:id="rId34" display="https://www.digikey.no/no/products/detail/kyocera-avx/08055A6R0CAT2A/1602729 "/>
-    <hyperlink ref="E48" r:id="rId35" display="https://www.digikey.no/no/products/detail/kemet/C0805C104K5RACTU/411169 "/>
-    <hyperlink ref="E49" r:id="rId36" display="https://www.digikey.no/no/products/detail/murata-electronics/GCJ21BR71H474KA12L/2783815 "/>
-    <hyperlink ref="E50" r:id="rId37" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL21B105KAFNNNE/3886724 "/>
-    <hyperlink ref="E51" r:id="rId38" display="https://www.digikey.no/no/products/detail/tdk-corporation/C2012X7R1C225K125AB/569046 "/>
-    <hyperlink ref="E52" r:id="rId39" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL21A475KAQNNNE/3886902 "/>
-    <hyperlink ref="E53" r:id="rId40" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL21A476MQYNNNE/3887510 "/>
-    <hyperlink ref="E55" r:id="rId41" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL31B106KAHNNNE/3887462"/>
-    <hyperlink ref="E56" r:id="rId42" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL31A226KAHNNNE/3888705 "/>
-    <hyperlink ref="E57" r:id="rId43" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL31A107MQHNNWE/10479833 "/>
-    <hyperlink ref="E59" r:id="rId44" display="https://www.digikey.no/no/products/detail/murata-electronics/GRM32ER60G337ME05L/6155746 "/>
-    <hyperlink ref="E62" r:id="rId45" display="https://www.digikey.no/no/products/detail/murata-electronics/LQM21PN1R5MC0D/1788280"/>
-    <hyperlink ref="E63" r:id="rId46" display="https://www.digikey.no/no/products/detail/murata-electronics/DFE201210U-2R2M-P2/7595453 "/>
-    <hyperlink ref="E64" r:id="rId47" display="https://www.digikey.no/no/products/detail/murata-electronics/LQM21PN3R3MGRD/4359175 "/>
+    <hyperlink ref="E16" r:id="rId11" display="https://www.digikey.no/no/products/detail/liteon/LTST-C193KGKT-5A/2356242 "/>
+    <hyperlink ref="E17" r:id="rId12" display="https://www.digikey.no/no/products/detail/liteon/LTST-C193KRKT-5A/2356244 "/>
+    <hyperlink ref="E18" r:id="rId13" display="https://www.digikey.no/no/products/detail/murata-electronics/XRCGB48M000F4M00R0/2368388 "/>
+    <hyperlink ref="E19" r:id="rId14" display="https://www.digikey.no/no/products/detail/connor-winfield/CWX813-100-0M/695541 "/>
+    <hyperlink ref="E20" r:id="rId15" display="https://www.digikey.no/no/products/detail/gigadevice-semiconductor-hk-limited/GD25F128FS2GR/20531633 "/>
+    <hyperlink ref="E21" r:id="rId16" display="https://www.digikey.no/no/products/detail/texas-instruments/TPS54294PWP/2812688 "/>
+    <hyperlink ref="E22" r:id="rId17" display="https://www.digikey.no/no/products/detail/issi-integrated-silicon-solution-inc/IS66WVH16M8DBLL-100B1LI/6202025 "/>
+    <hyperlink ref="E27" r:id="rId18" display="https://www.digikey.no/no/products/detail/amd/XC7A100T-2FTG256I/3925791?s=N4IgTCBcDaIBoGEDsBBAjABgwFQLRgDFsBxMAVgDYBJEAXQF8g "/>
+    <hyperlink ref="E28" r:id="rId19" display="https://www.digikey.no/en/products/detail/amphenol-cs-commercial-products/L77HDE15SD1CH4RHNVGA/25816614 "/>
+    <hyperlink ref="E33" r:id="rId20" display="https://www.digikey.no/no/products/detail/stackpole-electronics-inc/RMCF0805JT47R0/1757848 "/>
+    <hyperlink ref="E34" r:id="rId21" display="https://www.digikey.no/no/products/detail/panasonic-electronic-components/ERA-6AEB101V/1465724 "/>
+    <hyperlink ref="E35" r:id="rId22" display="https://www.digikey.no/no/products/detail/vishay-dale/CRCW0805270RFKEAC/7922379  "/>
+    <hyperlink ref="E36" r:id="rId23" display="https://www.digikey.no/no/products/detail/stackpole-electronics-inc/RMCF0805FT330R/1760484"/>
+    <hyperlink ref="E37" r:id="rId24" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-07536RL/728026 "/>
+    <hyperlink ref="E38" r:id="rId25" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-072K4L/727690"/>
+    <hyperlink ref="E39" r:id="rId26" display="https://www.digikey.no/no/products/detail/vishay-dale/CRCW08054K70FKEAC/7928553 "/>
+    <hyperlink ref="E40" r:id="rId27" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-076K81L/728068 "/>
+    <hyperlink ref="E41" r:id="rId28" display="https://www.digikey.no/no/products/detail/susumu/RR1220P-103-D/432315 "/>
+    <hyperlink ref="E42" r:id="rId29" display="https://www.digikey.no/no/products/detail/stackpole-electronics-inc/RMCF0805FT22K1/1760211 "/>
+    <hyperlink ref="E43" r:id="rId30" display="https://www.digikey.no/no/products/detail/vishay-dale/CRCW080530K1FKEA/1175804 "/>
+    <hyperlink ref="E44" r:id="rId31" display="https://www.digikey.no/no/products/detail/panasonic-electronic-components/ERA-6AEB7322V/2025832 "/>
+    <hyperlink ref="E45" r:id="rId32" display="https://www.digikey.no/no/products/detail/susumu/RG2012P-104-B-T5/1240656 "/>
+    <hyperlink ref="E46" r:id="rId33" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-07124KL/727580 "/>
+    <hyperlink ref="E49" r:id="rId34" display="https://www.digikey.no/no/products/detail/kyocera-avx/08055A6R0CAT2A/1602729 "/>
+    <hyperlink ref="E50" r:id="rId35" display="https://www.digikey.no/no/products/detail/kemet/C0805C104K5RACTU/411169 "/>
+    <hyperlink ref="E51" r:id="rId36" display="https://www.digikey.no/no/products/detail/murata-electronics/GCJ21BR71H474KA12L/2783815 "/>
+    <hyperlink ref="E52" r:id="rId37" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL21B105KAFNNNE/3886724 "/>
+    <hyperlink ref="E53" r:id="rId38" display="https://www.digikey.no/no/products/detail/tdk-corporation/C2012X7R1C225K125AB/569046 "/>
+    <hyperlink ref="E54" r:id="rId39" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL21A475KAQNNNE/3886902 "/>
+    <hyperlink ref="E55" r:id="rId40" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL21A476MQYNNNE/3887510 "/>
+    <hyperlink ref="E57" r:id="rId41" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL31B106KAHNNNE/3887462"/>
+    <hyperlink ref="E58" r:id="rId42" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL31A226KAHNNNE/3888705 "/>
+    <hyperlink ref="E59" r:id="rId43" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL31A107MQHNNWE/10479833 "/>
+    <hyperlink ref="E61" r:id="rId44" display="https://www.digikey.no/no/products/detail/murata-electronics/GRM32ER60G337ME05L/6155746 "/>
+    <hyperlink ref="E64" r:id="rId45" display="https://www.digikey.no/no/products/detail/murata-electronics/LQM21PN1R5MC0D/1788280"/>
+    <hyperlink ref="E65" r:id="rId46" display="https://www.digikey.no/no/products/detail/murata-electronics/DFE201210U-2R2M-P2/7595453 "/>
+    <hyperlink ref="E66" r:id="rId47" display="https://www.digikey.no/no/products/detail/murata-electronics/LQM21PN3R3MGRD/4359175 "/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
docs: latest version of Handleliste-hardware
</commit_message>
<xml_diff>
--- a/Handleliste-hardware.xlsx
+++ b/Handleliste-hardware.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="176">
   <si>
     <t xml:space="preserve">Komponent</t>
   </si>
@@ -52,6 +52,9 @@
     <t xml:space="preserve">Sendt inn</t>
   </si>
   <si>
+    <t xml:space="preserve">Faktisk kjøpeantall</t>
+  </si>
+  <si>
     <t xml:space="preserve">MCU</t>
   </si>
   <si>
@@ -356,6 +359,12 @@
   </si>
   <si>
     <t xml:space="preserve">Motstander</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12ohm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.no/en/products/detail/yageo/RC0805JR-0712RL/728249</t>
   </si>
   <si>
     <t xml:space="preserve">47ohm</t>
@@ -549,7 +558,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00\ %"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -582,18 +591,31 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF81D41A"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBF0041"/>
+        <bgColor rgb="FF800080"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -639,7 +661,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -648,7 +670,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -660,7 +690,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -702,7 +732,7 @@
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FFBF0041"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFC0C0C0"/>
       <rgbColor rgb="FF808080"/>
@@ -732,7 +762,7 @@
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FF81D41A"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
@@ -928,7 +958,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:K68"/>
+  <dimension ref="A2:M69"/>
   <sheetFormatPr defaultColWidth="8.55859375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.11"/>
@@ -938,7 +968,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="33.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="5.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="5.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="6.67"/>
   </cols>
@@ -962,7 +992,7 @@
       <c r="G2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="I2" s="1" t="s">
@@ -974,19 +1004,22 @@
       <c r="K2" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="M2" s="0" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="2" t="s">
         <v>13</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>1</v>
@@ -995,7 +1028,7 @@
         <f aca="false">F3*3</f>
         <v>3</v>
       </c>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I3" s="1" t="n">
@@ -1005,23 +1038,27 @@
         <f aca="false">H3*I3</f>
         <v>521.1</v>
       </c>
-      <c r="K3" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K3" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M3" s="1" t="n">
+        <f aca="false">H3</f>
+        <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="2" t="s">
         <v>17</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>1</v>
@@ -1030,7 +1067,7 @@
         <f aca="false">F4*3</f>
         <v>3</v>
       </c>
-      <c r="H4" s="1" t="n">
+      <c r="H4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I4" s="1" t="n">
@@ -1040,23 +1077,23 @@
         <f aca="false">H4*I4</f>
         <v>87.09</v>
       </c>
-      <c r="K4" s="1" t="b">
+      <c r="K4" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="2" t="s">
         <v>20</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>1</v>
@@ -1065,7 +1102,7 @@
         <f aca="false">F5*3</f>
         <v>3</v>
       </c>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I5" s="1" t="n">
@@ -1075,23 +1112,23 @@
         <f aca="false">H5*I5</f>
         <v>30.27</v>
       </c>
-      <c r="K5" s="1" t="b">
+      <c r="K5" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>1492</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>23</v>
+      <c r="E6" s="3" t="s">
+        <v>24</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>1</v>
@@ -1100,7 +1137,7 @@
         <f aca="false">F6*3</f>
         <v>3</v>
       </c>
-      <c r="H6" s="1" t="n">
+      <c r="H6" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I6" s="1" t="n">
@@ -1110,23 +1147,23 @@
         <f aca="false">H6*I6</f>
         <v>90.15</v>
       </c>
-      <c r="K6" s="1" t="b">
+      <c r="K6" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" s="3" t="s">
         <v>27</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>28</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>1</v>
@@ -1135,7 +1172,7 @@
         <f aca="false">F7*3</f>
         <v>3</v>
       </c>
-      <c r="H7" s="1" t="n">
+      <c r="H7" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I7" s="1" t="n">
@@ -1145,23 +1182,23 @@
         <f aca="false">H7*I7</f>
         <v>112.77</v>
       </c>
-      <c r="K7" s="1" t="b">
+      <c r="K7" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="D8" s="6" t="s">
         <v>31</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>1</v>
@@ -1170,7 +1207,7 @@
         <f aca="false">F8*3</f>
         <v>3</v>
       </c>
-      <c r="H8" s="1" t="n">
+      <c r="H8" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I8" s="1" t="n">
@@ -1180,24 +1217,24 @@
         <f aca="false">H8*I8</f>
         <v>1627.08</v>
       </c>
-      <c r="K8" s="1" t="b">
+      <c r="K8" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
+      <c r="A9" s="7"/>
       <c r="B9" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E9" s="3" t="s">
         <v>35</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>1</v>
@@ -1206,7 +1243,7 @@
         <f aca="false">F9*3</f>
         <v>3</v>
       </c>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I9" s="1" t="n">
@@ -1216,23 +1253,27 @@
         <f aca="false">H9*I9</f>
         <v>15.9</v>
       </c>
-      <c r="K9" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K9" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M9" s="1" t="n">
+        <f aca="false">H9</f>
+        <v>3</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" s="6" t="s">
         <v>39</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>40</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>1</v>
@@ -1241,7 +1282,7 @@
         <f aca="false">F10*3</f>
         <v>3</v>
       </c>
-      <c r="H10" s="1" t="n">
+      <c r="H10" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I10" s="1" t="n">
@@ -1251,48 +1292,51 @@
         <f aca="false">H10*I10</f>
         <v>280.56</v>
       </c>
-      <c r="K10" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K10" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="1" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E11" s="3" t="s">
         <v>42</v>
       </c>
+      <c r="E11" s="5" t="s">
+        <v>43</v>
+      </c>
       <c r="F11" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J11" s="1" t="n">
         <f aca="false">H11*I11</f>
         <v>0</v>
       </c>
-      <c r="K11" s="1" t="b">
+      <c r="K11" s="4" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E12" s="7" t="s">
         <v>47</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>48</v>
       </c>
       <c r="F12" s="1" t="n">
         <v>1</v>
@@ -1301,7 +1345,7 @@
         <f aca="false">F12*3</f>
         <v>3</v>
       </c>
-      <c r="H12" s="1" t="n">
+      <c r="H12" s="2" t="n">
         <v>4</v>
       </c>
       <c r="I12" s="1" t="n">
@@ -1311,23 +1355,27 @@
         <f aca="false">H12*I12</f>
         <v>20.36</v>
       </c>
-      <c r="K12" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K12" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M12" s="1" t="n">
+        <f aca="false">H12</f>
+        <v>4</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E13" s="7" t="s">
         <v>51</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>52</v>
       </c>
       <c r="F13" s="1" t="n">
         <v>2</v>
@@ -1336,7 +1384,7 @@
         <f aca="false">F13*3</f>
         <v>6</v>
       </c>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="2" t="n">
         <v>8</v>
       </c>
       <c r="I13" s="1" t="n">
@@ -1346,23 +1394,27 @@
         <f aca="false">H13*I13</f>
         <v>231.44</v>
       </c>
-      <c r="K13" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K13" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M13" s="1" t="n">
+        <f aca="false">H13</f>
+        <v>8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F14" s="1" t="n">
         <v>4</v>
@@ -1371,7 +1423,7 @@
         <f aca="false">F14*3</f>
         <v>12</v>
       </c>
-      <c r="H14" s="1" t="n">
+      <c r="H14" s="2" t="n">
         <v>14</v>
       </c>
       <c r="I14" s="1" t="n">
@@ -1381,23 +1433,27 @@
         <f aca="false">H14*I14</f>
         <v>243.88</v>
       </c>
-      <c r="K14" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K14" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M14" s="1" t="n">
+        <f aca="false">H14</f>
+        <v>14</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F15" s="1" t="n">
         <v>2</v>
@@ -1406,7 +1462,7 @@
         <f aca="false">F15*3</f>
         <v>6</v>
       </c>
-      <c r="H15" s="1" t="n">
+      <c r="H15" s="2" t="n">
         <v>8</v>
       </c>
       <c r="I15" s="1" t="n">
@@ -1416,23 +1472,26 @@
         <f aca="false">H15*I15</f>
         <v>61.12</v>
       </c>
-      <c r="K15" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K15" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M15" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E16" s="3" t="s">
         <v>63</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>64</v>
       </c>
       <c r="F16" s="1" t="n">
         <v>3</v>
@@ -1441,7 +1500,7 @@
         <f aca="false">F16*3</f>
         <v>9</v>
       </c>
-      <c r="H16" s="1" t="n">
+      <c r="H16" s="2" t="n">
         <v>12</v>
       </c>
       <c r="I16" s="1" t="n">
@@ -1451,23 +1510,27 @@
         <f aca="false">H16*I16</f>
         <v>24.48</v>
       </c>
-      <c r="K16" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K16" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M16" s="1" t="n">
+        <f aca="false">H16</f>
+        <v>12</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E17" s="3" t="s">
         <v>66</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>67</v>
       </c>
       <c r="F17" s="1" t="n">
         <v>2</v>
@@ -1476,7 +1539,7 @@
         <f aca="false">F17*3</f>
         <v>6</v>
       </c>
-      <c r="H17" s="1" t="n">
+      <c r="H17" s="2" t="n">
         <v>8</v>
       </c>
       <c r="I17" s="1" t="n">
@@ -1486,23 +1549,27 @@
         <f aca="false">H17*I17</f>
         <v>13.84</v>
       </c>
-      <c r="K17" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K17" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M17" s="1" t="n">
+        <f aca="false">H17</f>
+        <v>8</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E18" s="3" t="s">
         <v>70</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>71</v>
       </c>
       <c r="F18" s="1" t="n">
         <v>1</v>
@@ -1511,7 +1578,7 @@
         <f aca="false">F18*3</f>
         <v>3</v>
       </c>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="2" t="n">
         <v>4</v>
       </c>
       <c r="I18" s="1" t="n">
@@ -1521,23 +1588,27 @@
         <f aca="false">H18*I18</f>
         <v>12.24</v>
       </c>
-      <c r="K18" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K18" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M18" s="1" t="n">
+        <f aca="false">H18</f>
+        <v>4</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E19" s="3" t="s">
         <v>74</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="F19" s="1" t="n">
         <v>1</v>
@@ -1546,7 +1617,7 @@
         <f aca="false">F19*3</f>
         <v>3</v>
       </c>
-      <c r="H19" s="1" t="n">
+      <c r="H19" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I19" s="1" t="n">
@@ -1556,23 +1627,27 @@
         <f aca="false">H19*I19</f>
         <v>155.88</v>
       </c>
-      <c r="K19" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K19" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M19" s="1" t="n">
+        <f aca="false">H19</f>
+        <v>3</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E20" s="3" t="s">
         <v>78</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>79</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>1</v>
@@ -1581,7 +1656,7 @@
         <f aca="false">F20*3</f>
         <v>3</v>
       </c>
-      <c r="H20" s="1" t="n">
+      <c r="H20" s="2" t="n">
         <v>4</v>
       </c>
       <c r="I20" s="1" t="n">
@@ -1591,23 +1666,27 @@
         <f aca="false">H20*I20</f>
         <v>152.4</v>
       </c>
-      <c r="K20" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K20" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M20" s="1" t="n">
+        <f aca="false">H20</f>
+        <v>4</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="E21" s="3" t="s">
         <v>81</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>82</v>
       </c>
       <c r="F21" s="1" t="n">
         <v>2</v>
@@ -1616,7 +1695,7 @@
         <f aca="false">F21*3</f>
         <v>6</v>
       </c>
-      <c r="H21" s="1" t="n">
+      <c r="H21" s="2" t="n">
         <v>7</v>
       </c>
       <c r="I21" s="1" t="n">
@@ -1626,23 +1705,27 @@
         <f aca="false">H21*I21</f>
         <v>232.47</v>
       </c>
-      <c r="K21" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K21" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M21" s="1" t="n">
+        <f aca="false">H21</f>
+        <v>7</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="E22" s="3" t="s">
         <v>85</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>86</v>
       </c>
       <c r="F22" s="1" t="n">
         <v>1</v>
@@ -1651,7 +1734,7 @@
         <f aca="false">F22*3</f>
         <v>3</v>
       </c>
-      <c r="H22" s="1" t="n">
+      <c r="H22" s="2" t="n">
         <v>5</v>
       </c>
       <c r="I22" s="1" t="n">
@@ -1661,23 +1744,27 @@
         <f aca="false">H22*I22</f>
         <v>244.5</v>
       </c>
-      <c r="K22" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K22" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M22" s="1" t="n">
+        <f aca="false">H22</f>
+        <v>5</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F23" s="1" t="n">
         <v>1</v>
@@ -1686,7 +1773,7 @@
         <f aca="false">F23*3</f>
         <v>3</v>
       </c>
-      <c r="H23" s="1" t="n">
+      <c r="H23" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I23" s="1" t="n">
@@ -1696,23 +1783,26 @@
         <f aca="false">H23*I23</f>
         <v>9.78</v>
       </c>
-      <c r="K23" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K23" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M23" s="1" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="F24" s="1" t="n">
         <v>1</v>
@@ -1721,7 +1811,7 @@
         <f aca="false">F24*3</f>
         <v>3</v>
       </c>
-      <c r="H24" s="1" t="n">
+      <c r="H24" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I24" s="1" t="n">
@@ -1731,23 +1821,27 @@
         <f aca="false">H24*I24</f>
         <v>9.78</v>
       </c>
-      <c r="K24" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K24" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M24" s="1" t="n">
+        <f aca="false">H24</f>
+        <v>3</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F25" s="1" t="n">
         <v>1</v>
@@ -1756,7 +1850,7 @@
         <f aca="false">F25*3</f>
         <v>3</v>
       </c>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I25" s="1" t="n">
@@ -1766,23 +1860,26 @@
         <f aca="false">H25*I25</f>
         <v>23.22</v>
       </c>
-      <c r="K25" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K25" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M25" s="1" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D26" s="1" t="n">
         <v>61300811121</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F26" s="1" t="n">
         <v>1</v>
@@ -1791,7 +1888,7 @@
         <f aca="false">F26*3</f>
         <v>3</v>
       </c>
-      <c r="H26" s="1" t="n">
+      <c r="H26" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I26" s="1" t="n">
@@ -1801,23 +1898,26 @@
         <f aca="false">H26*I26</f>
         <v>11.01</v>
       </c>
-      <c r="K26" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K26" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M26" s="1" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="E27" s="3" t="s">
         <v>101</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>102</v>
       </c>
       <c r="F27" s="1" t="n">
         <v>1</v>
@@ -1826,7 +1926,7 @@
         <f aca="false">F27*3</f>
         <v>3</v>
       </c>
-      <c r="H27" s="1" t="n">
+      <c r="H27" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I27" s="1" t="n">
@@ -1836,23 +1936,27 @@
         <f aca="false">H27*I27</f>
         <v>5324.1</v>
       </c>
-      <c r="K27" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K27" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M27" s="1" t="n">
+        <f aca="false">H27</f>
+        <v>3</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D28" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="D28" s="10" t="s">
         <v>105</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>106</v>
       </c>
       <c r="F28" s="1" t="n">
         <v>1</v>
@@ -1861,7 +1965,7 @@
         <f aca="false">F28*3</f>
         <v>3</v>
       </c>
-      <c r="H28" s="1" t="n">
+      <c r="H28" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I28" s="1" t="n">
@@ -1871,23 +1975,27 @@
         <f aca="false">H28*I28</f>
         <v>57.15</v>
       </c>
-      <c r="K28" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K28" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M28" s="1" t="n">
+        <f aca="false">H28</f>
+        <v>3</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D29" s="1" t="n">
         <v>61300211121</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F29" s="1" t="n">
         <v>4</v>
@@ -1896,7 +2004,7 @@
         <f aca="false">F29*3</f>
         <v>12</v>
       </c>
-      <c r="H29" s="1" t="n">
+      <c r="H29" s="2" t="n">
         <v>12</v>
       </c>
       <c r="I29" s="1" t="n">
@@ -1906,23 +2014,26 @@
         <f aca="false">H29*I29</f>
         <v>14.64</v>
       </c>
-      <c r="K29" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K29" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M29" s="1" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F30" s="1" t="n">
         <v>4</v>
@@ -1931,7 +2042,7 @@
         <f aca="false">F30*3</f>
         <v>12</v>
       </c>
-      <c r="H30" s="1" t="n">
+      <c r="H30" s="2" t="n">
         <v>12</v>
       </c>
       <c r="I30" s="1" t="n">
@@ -1941,313 +2052,365 @@
         <f aca="false">H30*I30</f>
         <v>12.24</v>
       </c>
-      <c r="K30" s="1" t="b">
-        <f aca="false">FALSE()</f>
+      <c r="K30" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M30" s="1" t="n">
+        <f aca="false">H30</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G31" s="1" t="n">
+        <f aca="false">F31*3</f>
+        <v>0</v>
+      </c>
+      <c r="J31" s="1" t="n">
+        <f aca="false">H31*I31</f>
         <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
+      </c>
+      <c r="G32" s="1" t="n">
+        <f aca="false">F32*3</f>
+        <v>0</v>
+      </c>
+      <c r="J32" s="1" t="n">
+        <f aca="false">H32*I32</f>
+        <v>0</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C33" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E33" s="3" t="s">
-        <v>113</v>
+      <c r="E33" s="1" t="s">
+        <v>114</v>
       </c>
       <c r="F33" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G33" s="1" t="n">
         <f aca="false">F33*3</f>
-        <v>12</v>
-      </c>
-      <c r="H33" s="1" t="n">
-        <v>16</v>
+        <v>3</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>10</v>
       </c>
       <c r="I33" s="1" t="n">
-        <v>1.02</v>
+        <v>0.08</v>
       </c>
       <c r="J33" s="1" t="n">
         <f aca="false">H33*I33</f>
-        <v>16.32</v>
-      </c>
-      <c r="K33" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>0.8</v>
+      </c>
+      <c r="K33" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M33" s="0" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C34" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E34" s="3" t="s">
-        <v>115</v>
+      <c r="E34" s="5" t="s">
+        <v>116</v>
       </c>
       <c r="F34" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G34" s="1" t="n">
         <f aca="false">F34*3</f>
-        <v>6</v>
-      </c>
-      <c r="H34" s="1" t="n">
-        <v>8</v>
+        <v>12</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>16</v>
       </c>
       <c r="I34" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J34" s="1" t="n">
         <f aca="false">H34*I34</f>
-        <v>8.16</v>
-      </c>
-      <c r="K34" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>16.32</v>
+      </c>
+      <c r="K34" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M34" s="1" t="n">
+        <f aca="false">H34</f>
+        <v>16</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C35" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E35" s="3" t="s">
-        <v>117</v>
+      <c r="E35" s="5" t="s">
+        <v>118</v>
       </c>
       <c r="F35" s="1" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G35" s="1" t="n">
         <f aca="false">F35*3</f>
-        <v>42</v>
-      </c>
-      <c r="H35" s="1" t="n">
-        <v>50</v>
+        <v>6</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>8</v>
       </c>
       <c r="I35" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J35" s="1" t="n">
         <f aca="false">H35*I35</f>
-        <v>51</v>
-      </c>
-      <c r="K35" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>8.16</v>
+      </c>
+      <c r="K35" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M35" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C36" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E36" s="3" t="s">
-        <v>119</v>
+      <c r="E36" s="5" t="s">
+        <v>120</v>
       </c>
       <c r="F36" s="1" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G36" s="1" t="n">
         <f aca="false">F36*3</f>
-        <v>3</v>
-      </c>
-      <c r="H36" s="1" t="n">
-        <v>5</v>
+        <v>42</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>50</v>
       </c>
       <c r="I36" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J36" s="1" t="n">
         <f aca="false">H36*I36</f>
-        <v>5.1</v>
-      </c>
-      <c r="K36" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>51</v>
+      </c>
+      <c r="K36" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M36" s="1" t="n">
+        <f aca="false">H36</f>
+        <v>50</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C37" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E37" s="3" t="s">
-        <v>121</v>
+      <c r="E37" s="5" t="s">
+        <v>122</v>
       </c>
       <c r="F37" s="1" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="G37" s="1" t="n">
         <f aca="false">F37*3</f>
-        <v>45</v>
-      </c>
-      <c r="H37" s="1" t="n">
-        <v>55</v>
+        <v>3</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="I37" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J37" s="1" t="n">
         <f aca="false">H37*I37</f>
-        <v>56.1</v>
-      </c>
-      <c r="K37" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>5.1</v>
+      </c>
+      <c r="K37" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M37" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C38" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E38" s="3" t="s">
-        <v>123</v>
+      <c r="E38" s="5" t="s">
+        <v>124</v>
       </c>
       <c r="F38" s="1" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G38" s="1" t="n">
         <f aca="false">F38*3</f>
-        <v>3</v>
-      </c>
-      <c r="H38" s="1" t="n">
-        <v>5</v>
+        <v>45</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>55</v>
       </c>
       <c r="I38" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J38" s="1" t="n">
         <f aca="false">H38*I38</f>
-        <v>5.1</v>
-      </c>
-      <c r="K38" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>56.1</v>
+      </c>
+      <c r="K38" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M38" s="1" t="n">
+        <f aca="false">H38</f>
+        <v>55</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C39" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E39" s="3" t="s">
-        <v>125</v>
+      <c r="E39" s="5" t="s">
+        <v>126</v>
       </c>
       <c r="F39" s="1" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="G39" s="1" t="n">
         <f aca="false">F39*3</f>
-        <v>39</v>
-      </c>
-      <c r="H39" s="1" t="n">
-        <v>44</v>
+        <v>3</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="I39" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J39" s="1" t="n">
         <f aca="false">H39*I39</f>
-        <v>44.88</v>
-      </c>
-      <c r="K39" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>5.1</v>
+      </c>
+      <c r="K39" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M39" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C40" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E40" s="3" t="s">
-        <v>127</v>
+      <c r="E40" s="5" t="s">
+        <v>128</v>
       </c>
       <c r="F40" s="1" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="G40" s="1" t="n">
         <f aca="false">F40*3</f>
-        <v>3</v>
-      </c>
-      <c r="H40" s="1" t="n">
-        <v>5</v>
+        <v>39</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>44</v>
       </c>
       <c r="I40" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J40" s="1" t="n">
         <f aca="false">H40*I40</f>
-        <v>5.1</v>
-      </c>
-      <c r="K40" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>44.88</v>
+      </c>
+      <c r="K40" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M40" s="1" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C41" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E41" s="3" t="s">
-        <v>129</v>
+      <c r="E41" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="F41" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G41" s="1" t="n">
         <f aca="false">F41*3</f>
-        <v>12</v>
-      </c>
-      <c r="H41" s="1" t="n">
-        <v>15</v>
+        <v>3</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="I41" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J41" s="1" t="n">
         <f aca="false">H41*I41</f>
-        <v>15.3</v>
-      </c>
-      <c r="K41" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>5.1</v>
+      </c>
+      <c r="K41" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M41" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C42" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E42" s="3" t="s">
-        <v>131</v>
+      <c r="E42" s="5" t="s">
+        <v>132</v>
       </c>
       <c r="F42" s="1" t="n">
         <v>4</v>
@@ -2256,7 +2419,7 @@
         <f aca="false">F42*3</f>
         <v>12</v>
       </c>
-      <c r="H42" s="1" t="n">
+      <c r="H42" s="2" t="n">
         <v>15</v>
       </c>
       <c r="I42" s="1" t="n">
@@ -2266,52 +2429,60 @@
         <f aca="false">H42*I42</f>
         <v>15.3</v>
       </c>
-      <c r="K42" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K42" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M42" s="1" t="n">
+        <f aca="false">H42</f>
+        <v>15</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C43" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E43" s="3" t="s">
-        <v>133</v>
+      <c r="E43" s="5" t="s">
+        <v>134</v>
       </c>
       <c r="F43" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G43" s="1" t="n">
         <f aca="false">F43*3</f>
-        <v>3</v>
-      </c>
-      <c r="H43" s="1" t="n">
-        <v>5</v>
+        <v>12</v>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>15</v>
       </c>
       <c r="I43" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J43" s="1" t="n">
         <f aca="false">H43*I43</f>
-        <v>5.1</v>
-      </c>
-      <c r="K43" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>15.3</v>
+      </c>
+      <c r="K43" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M43" s="1" t="n">
+        <f aca="false">H43</f>
+        <v>15</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C44" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E44" s="3" t="s">
-        <v>135</v>
+      <c r="E44" s="5" t="s">
+        <v>136</v>
       </c>
       <c r="F44" s="1" t="n">
         <v>1</v>
@@ -2320,7 +2491,7 @@
         <f aca="false">F44*3</f>
         <v>3</v>
       </c>
-      <c r="H44" s="1" t="n">
+      <c r="H44" s="2" t="n">
         <v>5</v>
       </c>
       <c r="I44" s="1" t="n">
@@ -2330,153 +2501,170 @@
         <f aca="false">H44*I44</f>
         <v>5.1</v>
       </c>
-      <c r="K44" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K44" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M44" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C45" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E45" s="3" t="s">
-        <v>137</v>
+      <c r="E45" s="5" t="s">
+        <v>138</v>
       </c>
       <c r="F45" s="1" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G45" s="1" t="n">
         <f aca="false">F45*3</f>
-        <v>48</v>
-      </c>
-      <c r="H45" s="1" t="n">
-        <v>55</v>
+        <v>3</v>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="I45" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J45" s="1" t="n">
         <f aca="false">H45*I45</f>
-        <v>56.1</v>
-      </c>
-      <c r="K45" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>5.1</v>
+      </c>
+      <c r="K45" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M45" s="1" t="n">
+        <f aca="false">H45</f>
+        <v>5</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C46" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E46" s="3" t="s">
-        <v>139</v>
+      <c r="E46" s="5" t="s">
+        <v>140</v>
       </c>
       <c r="F46" s="1" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="G46" s="1" t="n">
         <f aca="false">F46*3</f>
-        <v>3</v>
-      </c>
-      <c r="H46" s="1" t="n">
-        <v>5</v>
+        <v>48</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>55</v>
       </c>
       <c r="I46" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="J46" s="1" t="n">
         <f aca="false">H46*I46</f>
+        <v>56.1</v>
+      </c>
+      <c r="K46" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M46" s="1" t="n">
+        <f aca="false">H46</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B47" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C47" s="1" t="n">
+        <v>805</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="F47" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="1" t="n">
+        <f aca="false">F47*3</f>
+        <v>3</v>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I47" s="1" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J47" s="1" t="n">
+        <f aca="false">H47*I47</f>
         <v>5.1</v>
       </c>
-      <c r="K46" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B48" s="1" t="s">
-        <v>140</v>
+      <c r="K47" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M47" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="C49" s="1" t="n">
-        <v>805</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="F49" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G49" s="1" t="n">
-        <f aca="false">F49*3</f>
-        <v>6</v>
-      </c>
-      <c r="H49" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="I49" s="1" t="n">
-        <v>2.04</v>
-      </c>
-      <c r="J49" s="1" t="n">
-        <f aca="false">H49*I49</f>
-        <v>16.32</v>
-      </c>
-      <c r="K49" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>143</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C50" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E50" s="3" t="s">
-        <v>144</v>
+      <c r="E50" s="5" t="s">
+        <v>145</v>
       </c>
       <c r="F50" s="1" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="G50" s="1" t="n">
         <f aca="false">F50*3</f>
-        <v>63</v>
-      </c>
-      <c r="H50" s="1" t="n">
-        <v>70</v>
+        <v>6</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>8</v>
       </c>
       <c r="I50" s="1" t="n">
-        <v>0.82</v>
+        <v>2.04</v>
       </c>
       <c r="J50" s="1" t="n">
         <f aca="false">H50*I50</f>
-        <v>57.4</v>
-      </c>
-      <c r="K50" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>16.32</v>
+      </c>
+      <c r="K50" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M50" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C51" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E51" s="3" t="s">
-        <v>146</v>
+      <c r="E51" s="5" t="s">
+        <v>147</v>
       </c>
       <c r="F51" s="1" t="n">
         <v>21</v>
@@ -2485,190 +2673,212 @@
         <f aca="false">F51*3</f>
         <v>63</v>
       </c>
-      <c r="H51" s="1" t="n">
+      <c r="H51" s="2" t="n">
         <v>70</v>
       </c>
       <c r="I51" s="1" t="n">
-        <v>2.65</v>
+        <v>0.82</v>
       </c>
       <c r="J51" s="1" t="n">
         <f aca="false">H51*I51</f>
-        <v>185.5</v>
-      </c>
-      <c r="K51" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>57.4</v>
+      </c>
+      <c r="K51" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M51" s="1" t="n">
+        <f aca="false">H51</f>
+        <v>70</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C52" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E52" s="3" t="s">
-        <v>148</v>
+      <c r="E52" s="5" t="s">
+        <v>149</v>
       </c>
       <c r="F52" s="1" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="G52" s="1" t="n">
         <f aca="false">F52*3</f>
-        <v>18</v>
-      </c>
-      <c r="H52" s="1" t="n">
-        <v>22</v>
+        <v>63</v>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>70</v>
       </c>
       <c r="I52" s="1" t="n">
-        <v>0.82</v>
+        <v>2.65</v>
       </c>
       <c r="J52" s="1" t="n">
         <f aca="false">H52*I52</f>
-        <v>18.04</v>
-      </c>
-      <c r="K52" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>185.5</v>
+      </c>
+      <c r="K52" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M52" s="1" t="n">
+        <f aca="false">H52</f>
+        <v>70</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C53" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E53" s="3" t="s">
-        <v>150</v>
+      <c r="E53" s="5" t="s">
+        <v>151</v>
       </c>
       <c r="F53" s="1" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G53" s="1" t="n">
         <f aca="false">F53*3</f>
-        <v>6</v>
-      </c>
-      <c r="H53" s="1" t="n">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>22</v>
       </c>
       <c r="I53" s="1" t="n">
-        <v>1.83</v>
+        <v>0.82</v>
       </c>
       <c r="J53" s="1" t="n">
         <f aca="false">H53*I53</f>
-        <v>14.64</v>
-      </c>
-      <c r="K53" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>18.04</v>
+      </c>
+      <c r="K53" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M53" s="1" t="n">
+        <f aca="false">H53</f>
+        <v>22</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C54" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E54" s="3" t="s">
-        <v>152</v>
+      <c r="E54" s="5" t="s">
+        <v>153</v>
       </c>
       <c r="F54" s="1" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G54" s="1" t="n">
         <f aca="false">F54*3</f>
-        <v>36</v>
-      </c>
-      <c r="H54" s="1" t="n">
-        <v>42</v>
+        <v>6</v>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>8</v>
       </c>
       <c r="I54" s="1" t="n">
-        <v>1.02</v>
+        <v>1.83</v>
       </c>
       <c r="J54" s="1" t="n">
         <f aca="false">H54*I54</f>
-        <v>42.84</v>
-      </c>
-      <c r="K54" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>14.64</v>
+      </c>
+      <c r="K54" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M54" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C55" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E55" s="3" t="s">
-        <v>154</v>
+      <c r="E55" s="5" t="s">
+        <v>155</v>
       </c>
       <c r="F55" s="1" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G55" s="1" t="n">
         <f aca="false">F55*3</f>
-        <v>12</v>
-      </c>
-      <c r="H55" s="1" t="n">
-        <v>15</v>
+        <v>36</v>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>42</v>
       </c>
       <c r="I55" s="1" t="n">
-        <v>1.32</v>
+        <v>1.02</v>
       </c>
       <c r="J55" s="1" t="n">
         <f aca="false">H55*I55</f>
+        <v>42.84</v>
+      </c>
+      <c r="K55" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M55" s="1" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B56" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C56" s="1" t="n">
+        <v>805</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="F56" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="G56" s="1" t="n">
+        <f aca="false">F56*3</f>
+        <v>12</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I56" s="1" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="J56" s="1" t="n">
+        <f aca="false">H56*I56</f>
         <v>19.8</v>
       </c>
-      <c r="K55" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B57" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="C57" s="1" t="n">
-        <v>1206</v>
-      </c>
-      <c r="E57" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="F57" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="G57" s="1" t="n">
-        <f aca="false">F57*3</f>
-        <v>24</v>
-      </c>
-      <c r="H57" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="I57" s="1" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="J57" s="1" t="n">
-        <f aca="false">H57*I57</f>
-        <v>22.96</v>
-      </c>
-      <c r="K57" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K56" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M56" s="1" t="n">
+        <f aca="false">H56</f>
+        <v>15</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C58" s="1" t="n">
         <v>1206</v>
       </c>
-      <c r="E58" s="3" t="s">
-        <v>158</v>
+      <c r="E58" s="5" t="s">
+        <v>159</v>
       </c>
       <c r="F58" s="1" t="n">
         <v>8</v>
@@ -2677,131 +2887,148 @@
         <f aca="false">F58*3</f>
         <v>24</v>
       </c>
-      <c r="H58" s="1" t="n">
+      <c r="H58" s="2" t="n">
         <v>28</v>
       </c>
       <c r="I58" s="1" t="n">
-        <v>0.92</v>
+        <v>0.82</v>
       </c>
       <c r="J58" s="1" t="n">
         <f aca="false">H58*I58</f>
-        <v>25.76</v>
-      </c>
-      <c r="K58" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>22.96</v>
+      </c>
+      <c r="K58" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M58" s="1" t="n">
+        <f aca="false">H58</f>
+        <v>28</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B59" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C59" s="1" t="n">
         <v>1206</v>
       </c>
-      <c r="E59" s="3" t="s">
-        <v>160</v>
+      <c r="E59" s="5" t="s">
+        <v>161</v>
       </c>
       <c r="F59" s="1" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G59" s="1" t="n">
         <f aca="false">F59*3</f>
-        <v>3</v>
-      </c>
-      <c r="H59" s="1" t="n">
-        <v>5</v>
+        <v>24</v>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>28</v>
       </c>
       <c r="I59" s="1" t="n">
-        <v>4.08</v>
+        <v>0.92</v>
       </c>
       <c r="J59" s="1" t="n">
         <f aca="false">H59*I59</f>
+        <v>25.76</v>
+      </c>
+      <c r="K59" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M59" s="1" t="n">
+        <f aca="false">H59</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B60" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C60" s="1" t="n">
+        <v>1206</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="F60" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="1" t="n">
+        <f aca="false">F60*3</f>
+        <v>3</v>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I60" s="1" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="J60" s="1" t="n">
+        <f aca="false">H60*I60</f>
         <v>20.4</v>
       </c>
-      <c r="K59" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B61" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="C61" s="1" t="n">
+      <c r="K60" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M60" s="1" t="n">
+        <f aca="false">H60</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B62" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C62" s="1" t="n">
         <v>1210</v>
       </c>
-      <c r="E61" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="F61" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G61" s="1" t="n">
-        <f aca="false">F61*3</f>
-        <v>3</v>
-      </c>
-      <c r="H61" s="1" t="n">
+      <c r="E62" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="F62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="1" t="n">
+        <f aca="false">F62*3</f>
+        <v>3</v>
+      </c>
+      <c r="H62" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="I61" s="1" t="n">
+      <c r="I62" s="1" t="n">
         <v>16.61</v>
       </c>
-      <c r="J61" s="1" t="n">
-        <f aca="false">H61*I61</f>
+      <c r="J62" s="1" t="n">
+        <f aca="false">H62*I62</f>
         <v>66.44</v>
       </c>
-      <c r="K61" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B63" s="1" t="s">
-        <v>163</v>
+      <c r="K62" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M62" s="1" t="n">
+        <f aca="false">H62</f>
+        <v>4</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="C64" s="1" t="n">
-        <v>805</v>
-      </c>
-      <c r="E64" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="F64" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G64" s="1" t="n">
-        <f aca="false">F64*3</f>
-        <v>6</v>
-      </c>
-      <c r="H64" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="I64" s="1" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="J64" s="1" t="n">
-        <f aca="false">H64*I64</f>
-        <v>13.84</v>
-      </c>
-      <c r="K64" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
+        <v>166</v>
+      </c>
+      <c r="K64" s="4"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C65" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E65" s="3" t="s">
-        <v>167</v>
+      <c r="E65" s="5" t="s">
+        <v>168</v>
       </c>
       <c r="F65" s="1" t="n">
         <v>2</v>
@@ -2810,70 +3037,117 @@
         <f aca="false">F65*3</f>
         <v>6</v>
       </c>
-      <c r="H65" s="1" t="n">
+      <c r="H65" s="2" t="n">
         <v>8</v>
       </c>
       <c r="I65" s="1" t="n">
-        <v>2.45</v>
+        <v>1.73</v>
       </c>
       <c r="J65" s="1" t="n">
         <f aca="false">H65*I65</f>
-        <v>19.6</v>
-      </c>
-      <c r="K65" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>13.84</v>
+      </c>
+      <c r="K65" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M65" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B66" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C66" s="1" t="n">
         <v>805</v>
       </c>
-      <c r="E66" s="3" t="s">
-        <v>169</v>
+      <c r="E66" s="5" t="s">
+        <v>170</v>
       </c>
       <c r="F66" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G66" s="1" t="n">
         <f aca="false">F66*3</f>
-        <v>3</v>
-      </c>
-      <c r="H66" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>8</v>
       </c>
       <c r="I66" s="1" t="n">
-        <v>1.73</v>
+        <v>2.45</v>
       </c>
       <c r="J66" s="1" t="n">
         <f aca="false">H66*I66</f>
+        <v>19.6</v>
+      </c>
+      <c r="K66" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M66" s="1" t="n">
+        <f aca="false">H66</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B67" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C67" s="1" t="n">
+        <v>805</v>
+      </c>
+      <c r="E67" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="F67" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="1" t="n">
+        <f aca="false">F67*3</f>
+        <v>3</v>
+      </c>
+      <c r="H67" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I67" s="1" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="J67" s="1" t="n">
+        <f aca="false">H67*I67</f>
         <v>8.65</v>
       </c>
-      <c r="K66" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E68" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="F68" s="1" t="n">
-        <f aca="false">SUM(F3:F66)</f>
-        <v>211</v>
-      </c>
-      <c r="I68" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="J68" s="1" t="n">
-        <f aca="false">SUM(J3:J67)</f>
-        <v>10445.4</v>
-      </c>
-      <c r="K68" s="1" t="s">
-        <v>172</v>
+      <c r="K67" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M67" s="1" t="n">
+        <f aca="false">H67</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E69" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="F69" s="1" t="n">
+        <f aca="false">SUM(F3:F67)</f>
+        <v>212</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="J69" s="1" t="n">
+        <f aca="false">SUM(J3:J68)</f>
+        <v>10446.2</v>
+      </c>
+      <c r="K69" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="M69" s="1" t="n">
+        <f aca="false">SUM(M3:M67)</f>
+        <v>802</v>
       </c>
     </row>
   </sheetData>
@@ -2897,34 +3171,34 @@
     <hyperlink ref="E22" r:id="rId17" display="https://www.digikey.no/no/products/detail/issi-integrated-silicon-solution-inc/IS66WVH16M8DBLL-100B1LI/6202025 "/>
     <hyperlink ref="E27" r:id="rId18" display="https://www.digikey.no/no/products/detail/amd/XC7A100T-2FTG256I/3925791?s=N4IgTCBcDaIBoGEDsBBAjABgwFQLRgDFsBxMAVgDYBJEAXQF8g "/>
     <hyperlink ref="E28" r:id="rId19" display="https://www.digikey.no/en/products/detail/amphenol-cs-commercial-products/L77HDE15SD1CH4RHNVGA/25816614 "/>
-    <hyperlink ref="E33" r:id="rId20" display="https://www.digikey.no/no/products/detail/stackpole-electronics-inc/RMCF0805JT47R0/1757848 "/>
-    <hyperlink ref="E34" r:id="rId21" display="https://www.digikey.no/no/products/detail/panasonic-electronic-components/ERA-6AEB101V/1465724 "/>
-    <hyperlink ref="E35" r:id="rId22" display="https://www.digikey.no/no/products/detail/vishay-dale/CRCW0805270RFKEAC/7922379  "/>
-    <hyperlink ref="E36" r:id="rId23" display="https://www.digikey.no/no/products/detail/stackpole-electronics-inc/RMCF0805FT330R/1760484"/>
-    <hyperlink ref="E37" r:id="rId24" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-07536RL/728026 "/>
-    <hyperlink ref="E38" r:id="rId25" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-072K4L/727690"/>
-    <hyperlink ref="E39" r:id="rId26" display="https://www.digikey.no/no/products/detail/vishay-dale/CRCW08054K70FKEAC/7928553 "/>
-    <hyperlink ref="E40" r:id="rId27" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-076K81L/728068 "/>
-    <hyperlink ref="E41" r:id="rId28" display="https://www.digikey.no/no/products/detail/susumu/RR1220P-103-D/432315 "/>
-    <hyperlink ref="E42" r:id="rId29" display="https://www.digikey.no/no/products/detail/stackpole-electronics-inc/RMCF0805FT22K1/1760211 "/>
-    <hyperlink ref="E43" r:id="rId30" display="https://www.digikey.no/no/products/detail/vishay-dale/CRCW080530K1FKEA/1175804 "/>
-    <hyperlink ref="E44" r:id="rId31" display="https://www.digikey.no/no/products/detail/panasonic-electronic-components/ERA-6AEB7322V/2025832 "/>
-    <hyperlink ref="E45" r:id="rId32" display="https://www.digikey.no/no/products/detail/susumu/RG2012P-104-B-T5/1240656 "/>
-    <hyperlink ref="E46" r:id="rId33" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-07124KL/727580 "/>
-    <hyperlink ref="E49" r:id="rId34" display="https://www.digikey.no/no/products/detail/kyocera-avx/08055A6R0CAT2A/1602729 "/>
-    <hyperlink ref="E50" r:id="rId35" display="https://www.digikey.no/no/products/detail/kemet/C0805C104K5RACTU/411169 "/>
-    <hyperlink ref="E51" r:id="rId36" display="https://www.digikey.no/no/products/detail/murata-electronics/GCJ21BR71H474KA12L/2783815 "/>
-    <hyperlink ref="E52" r:id="rId37" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL21B105KAFNNNE/3886724 "/>
-    <hyperlink ref="E53" r:id="rId38" display="https://www.digikey.no/no/products/detail/tdk-corporation/C2012X7R1C225K125AB/569046 "/>
-    <hyperlink ref="E54" r:id="rId39" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL21A475KAQNNNE/3886902 "/>
-    <hyperlink ref="E55" r:id="rId40" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL21A476MQYNNNE/3887510 "/>
-    <hyperlink ref="E57" r:id="rId41" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL31B106KAHNNNE/3887462"/>
-    <hyperlink ref="E58" r:id="rId42" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL31A226KAHNNNE/3888705 "/>
-    <hyperlink ref="E59" r:id="rId43" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL31A107MQHNNWE/10479833 "/>
-    <hyperlink ref="E61" r:id="rId44" display="https://www.digikey.no/no/products/detail/murata-electronics/GRM32ER60G337ME05L/6155746 "/>
-    <hyperlink ref="E64" r:id="rId45" display="https://www.digikey.no/no/products/detail/murata-electronics/LQM21PN1R5MC0D/1788280"/>
-    <hyperlink ref="E65" r:id="rId46" display="https://www.digikey.no/no/products/detail/murata-electronics/DFE201210U-2R2M-P2/7595453 "/>
-    <hyperlink ref="E66" r:id="rId47" display="https://www.digikey.no/no/products/detail/murata-electronics/LQM21PN3R3MGRD/4359175 "/>
+    <hyperlink ref="E34" r:id="rId20" display="https://www.digikey.no/no/products/detail/stackpole-electronics-inc/RMCF0805JT47R0/1757848 "/>
+    <hyperlink ref="E35" r:id="rId21" display="https://www.digikey.no/no/products/detail/panasonic-electronic-components/ERA-6AEB101V/1465724 "/>
+    <hyperlink ref="E36" r:id="rId22" display="https://www.digikey.no/no/products/detail/vishay-dale/CRCW0805270RFKEAC/7922379  "/>
+    <hyperlink ref="E37" r:id="rId23" display="https://www.digikey.no/no/products/detail/stackpole-electronics-inc/RMCF0805FT330R/1760484"/>
+    <hyperlink ref="E38" r:id="rId24" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-07536RL/728026 "/>
+    <hyperlink ref="E39" r:id="rId25" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-072K4L/727690"/>
+    <hyperlink ref="E40" r:id="rId26" display="https://www.digikey.no/no/products/detail/vishay-dale/CRCW08054K70FKEAC/7928553 "/>
+    <hyperlink ref="E41" r:id="rId27" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-076K81L/728068 "/>
+    <hyperlink ref="E42" r:id="rId28" display="https://www.digikey.no/no/products/detail/susumu/RR1220P-103-D/432315 "/>
+    <hyperlink ref="E43" r:id="rId29" display="https://www.digikey.no/no/products/detail/stackpole-electronics-inc/RMCF0805FT22K1/1760211 "/>
+    <hyperlink ref="E44" r:id="rId30" display="https://www.digikey.no/no/products/detail/vishay-dale/CRCW080530K1FKEA/1175804 "/>
+    <hyperlink ref="E45" r:id="rId31" display="https://www.digikey.no/no/products/detail/panasonic-electronic-components/ERA-6AEB7322V/2025832 "/>
+    <hyperlink ref="E46" r:id="rId32" display="https://www.digikey.no/no/products/detail/susumu/RG2012P-104-B-T5/1240656 "/>
+    <hyperlink ref="E47" r:id="rId33" display="https://www.digikey.no/no/products/detail/yageo/RC0805FR-07124KL/727580 "/>
+    <hyperlink ref="E50" r:id="rId34" display="https://www.digikey.no/no/products/detail/kyocera-avx/08055A6R0CAT2A/1602729 "/>
+    <hyperlink ref="E51" r:id="rId35" display="https://www.digikey.no/no/products/detail/kemet/C0805C104K5RACTU/411169 "/>
+    <hyperlink ref="E52" r:id="rId36" display="https://www.digikey.no/no/products/detail/murata-electronics/GCJ21BR71H474KA12L/2783815 "/>
+    <hyperlink ref="E53" r:id="rId37" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL21B105KAFNNNE/3886724 "/>
+    <hyperlink ref="E54" r:id="rId38" display="https://www.digikey.no/no/products/detail/tdk-corporation/C2012X7R1C225K125AB/569046 "/>
+    <hyperlink ref="E55" r:id="rId39" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL21A475KAQNNNE/3886902 "/>
+    <hyperlink ref="E56" r:id="rId40" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL21A476MQYNNNE/3887510 "/>
+    <hyperlink ref="E58" r:id="rId41" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL31B106KAHNNNE/3887462"/>
+    <hyperlink ref="E59" r:id="rId42" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL31A226KAHNNNE/3888705 "/>
+    <hyperlink ref="E60" r:id="rId43" display="https://www.digikey.no/no/products/detail/samsung-electro-mechanics/CL31A107MQHNNWE/10479833 "/>
+    <hyperlink ref="E62" r:id="rId44" display="https://www.digikey.no/no/products/detail/murata-electronics/GRM32ER60G337ME05L/6155746 "/>
+    <hyperlink ref="E65" r:id="rId45" display="https://www.digikey.no/no/products/detail/murata-electronics/LQM21PN1R5MC0D/1788280"/>
+    <hyperlink ref="E66" r:id="rId46" display="https://www.digikey.no/no/products/detail/murata-electronics/DFE201210U-2R2M-P2/7595453 "/>
+    <hyperlink ref="E67" r:id="rId47" display="https://www.digikey.no/no/products/detail/murata-electronics/LQM21PN3R3MGRD/4359175 "/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>